<commit_message>
End year propagation fix, Grid Emissions on Results page, retrained ML models, and UI improvements
- Fix endYear not propagating from frontend to backend generation pipeline
- Fix get_year_range() to respect user-selected endYear instead of using max ABM upload year
- Remove Grid Emission Rates from Results page (keep only Grid Emissions)
- Add Grid Emissions chart component and generated data files
- Widen End Year dropdown for better display
- Retrain GA ML models with AI feedback loop
- Update static R1/R2/R3 fallback data and pregenerated state files
- Add ABM manifest, GA 2033 ABM data, and generated output files
- Add backend utility scripts for MOVES5 data fixes, grid emissions, and pipeline

Co-Authored-By: Claude Opus 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/backend/Combined_sheet_output_speed/GA/GA_2040_ABM.xlsx
+++ b/backend/Combined_sheet_output_speed/GA/GA_2040_ABM.xlsx
@@ -1,32 +1,32 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="tract=13121001001" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="tract=13121001002" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="tract=13121001201" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="tract=13121001202" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet name="tract=13121001800" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet name="tract=13121001900" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet name="tract=13121002100" sheetId="7" state="visible" r:id="rId7"/>
-    <sheet name="tract=13121002600" sheetId="8" state="visible" r:id="rId8"/>
-    <sheet name="tract=13121002800" sheetId="9" state="visible" r:id="rId9"/>
-    <sheet name="tract=13121003500" sheetId="10" state="visible" r:id="rId10"/>
-    <sheet name="tract=13121003600" sheetId="11" state="visible" r:id="rId11"/>
-    <sheet name="tract=13121003800" sheetId="12" state="visible" r:id="rId12"/>
-    <sheet name="tract=13121004300" sheetId="13" state="visible" r:id="rId13"/>
-    <sheet name="tract=13121004400" sheetId="14" state="visible" r:id="rId14"/>
-    <sheet name="tract=13121004800" sheetId="15" state="visible" r:id="rId15"/>
-    <sheet name="tract=13121004900" sheetId="16" state="visible" r:id="rId16"/>
-    <sheet name="tract=13121005800" sheetId="17" state="visible" r:id="rId17"/>
-    <sheet name="tract=13121011800" sheetId="18" state="visible" r:id="rId18"/>
-    <sheet name="tract=13121011900" sheetId="19" state="visible" r:id="rId19"/>
-    <sheet name="tract=13121012000" sheetId="20" state="visible" r:id="rId20"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="tract=13121001001" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="tract=13121001002" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="tract=13121001201" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="tract=13121001202" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="tract=13121001800" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="tract=13121001900" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="tract=13121002100" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="tract=13121002600" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="tract=13121002800" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="tract=13121003500" sheetId="10" state="visible" r:id="rId10"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="tract=13121003600" sheetId="11" state="visible" r:id="rId11"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="tract=13121003800" sheetId="12" state="visible" r:id="rId12"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="tract=13121004300" sheetId="13" state="visible" r:id="rId13"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="tract=13121004400" sheetId="14" state="visible" r:id="rId14"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="tract=13121004800" sheetId="15" state="visible" r:id="rId15"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="tract=13121004900" sheetId="16" state="visible" r:id="rId16"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="tract=13121005800" sheetId="17" state="visible" r:id="rId17"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="tract=13121011800" sheetId="18" state="visible" r:id="rId18"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="tract=13121011900" sheetId="19" state="visible" r:id="rId19"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="tract=13121012000" sheetId="20" state="visible" r:id="rId20"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -4966,10 +4966,10 @@
         <v>52.90068159688413</v>
       </c>
       <c r="D70" t="n">
-        <v>22.13704175034878</v>
+        <v>22.13704175034877</v>
       </c>
       <c r="E70" t="n">
-        <v>22.13704175034878</v>
+        <v>22.13704175034877</v>
       </c>
       <c r="F70" t="n">
         <v>52.90068159688413</v>
@@ -4993,10 +4993,10 @@
         <v>52.90068159688413</v>
       </c>
       <c r="D71" t="n">
-        <v>22.13704175034878</v>
+        <v>22.13704175034877</v>
       </c>
       <c r="E71" t="n">
-        <v>22.13704175034878</v>
+        <v>22.13704175034877</v>
       </c>
       <c r="F71" t="n">
         <v>52.90068159688413</v>
@@ -5020,10 +5020,10 @@
         <v>52.90068159688413</v>
       </c>
       <c r="D72" t="n">
-        <v>22.13704175034878</v>
+        <v>22.13704175034877</v>
       </c>
       <c r="E72" t="n">
-        <v>22.13704175034878</v>
+        <v>22.13704175034877</v>
       </c>
       <c r="F72" t="n">
         <v>52.90068159688413</v>
@@ -5047,10 +5047,10 @@
         <v>52.90068159688413</v>
       </c>
       <c r="D73" t="n">
-        <v>22.13704175034878</v>
+        <v>22.13704175034877</v>
       </c>
       <c r="E73" t="n">
-        <v>22.13704175034878</v>
+        <v>22.13704175034877</v>
       </c>
       <c r="F73" t="n">
         <v>52.90068159688413</v>
@@ -5074,10 +5074,10 @@
         <v>52.90068159688413</v>
       </c>
       <c r="D74" t="n">
-        <v>22.13704175034878</v>
+        <v>22.13704175034877</v>
       </c>
       <c r="E74" t="n">
-        <v>22.13704175034878</v>
+        <v>22.13704175034877</v>
       </c>
       <c r="F74" t="n">
         <v>52.90068159688413</v>
@@ -5101,10 +5101,10 @@
         <v>52.90068159688413</v>
       </c>
       <c r="D75" t="n">
-        <v>22.13704175034878</v>
+        <v>22.13704175034877</v>
       </c>
       <c r="E75" t="n">
-        <v>22.13704175034878</v>
+        <v>22.13704175034877</v>
       </c>
       <c r="F75" t="n">
         <v>52.90068159688413</v>
@@ -5128,10 +5128,10 @@
         <v>52.90068159688413</v>
       </c>
       <c r="D76" t="n">
-        <v>22.13704175034878</v>
+        <v>22.13704175034877</v>
       </c>
       <c r="E76" t="n">
-        <v>22.13704175034878</v>
+        <v>22.13704175034877</v>
       </c>
       <c r="F76" t="n">
         <v>52.90068159688413</v>
@@ -5155,10 +5155,10 @@
         <v>52.90068159688413</v>
       </c>
       <c r="D77" t="n">
-        <v>22.13704175034878</v>
+        <v>22.13704175034877</v>
       </c>
       <c r="E77" t="n">
-        <v>22.13704175034878</v>
+        <v>22.13704175034877</v>
       </c>
       <c r="F77" t="n">
         <v>52.90068159688413</v>
@@ -5182,10 +5182,10 @@
         <v>52.90068159688413</v>
       </c>
       <c r="D78" t="n">
-        <v>22.13704175034878</v>
+        <v>22.13704175034877</v>
       </c>
       <c r="E78" t="n">
-        <v>22.13704175034878</v>
+        <v>22.13704175034877</v>
       </c>
       <c r="F78" t="n">
         <v>52.90068159688413</v>
@@ -5209,10 +5209,10 @@
         <v>52.90068159688413</v>
       </c>
       <c r="D79" t="n">
-        <v>22.13704175034878</v>
+        <v>22.13704175034877</v>
       </c>
       <c r="E79" t="n">
-        <v>22.13704175034878</v>
+        <v>22.13704175034877</v>
       </c>
       <c r="F79" t="n">
         <v>52.90068159688413</v>
@@ -5236,10 +5236,10 @@
         <v>52.90068159688413</v>
       </c>
       <c r="D80" t="n">
-        <v>22.13704175034878</v>
+        <v>22.13704175034877</v>
       </c>
       <c r="E80" t="n">
-        <v>22.13704175034878</v>
+        <v>22.13704175034877</v>
       </c>
       <c r="F80" t="n">
         <v>52.90068159688413</v>
@@ -5263,10 +5263,10 @@
         <v>52.90068159688413</v>
       </c>
       <c r="D81" t="n">
-        <v>22.13704175034878</v>
+        <v>22.13704175034877</v>
       </c>
       <c r="E81" t="n">
-        <v>22.13704175034878</v>
+        <v>22.13704175034877</v>
       </c>
       <c r="F81" t="n">
         <v>52.90068159688413</v>
@@ -8416,16 +8416,16 @@
         <v>20.72818791946309</v>
       </c>
       <c r="D2" t="n">
-        <v>22.3309425629695</v>
+        <v>22.33094256296949</v>
       </c>
       <c r="E2" t="n">
-        <v>22.3309425629695</v>
+        <v>22.33094256296949</v>
       </c>
       <c r="F2" t="n">
         <v>20.72818791946309</v>
       </c>
       <c r="G2" t="n">
-        <v>0.9282271834703389</v>
+        <v>0.9282271834703392</v>
       </c>
     </row>
     <row r="3">
@@ -8443,16 +8443,16 @@
         <v>20.72818791946309</v>
       </c>
       <c r="D3" t="n">
-        <v>22.3309425629695</v>
+        <v>22.33094256296949</v>
       </c>
       <c r="E3" t="n">
-        <v>22.3309425629695</v>
+        <v>22.33094256296949</v>
       </c>
       <c r="F3" t="n">
         <v>20.72818791946309</v>
       </c>
       <c r="G3" t="n">
-        <v>0.9282271834703389</v>
+        <v>0.9282271834703392</v>
       </c>
     </row>
     <row r="4">
@@ -8470,16 +8470,16 @@
         <v>20.72818791946309</v>
       </c>
       <c r="D4" t="n">
-        <v>22.3309425629695</v>
+        <v>22.33094256296949</v>
       </c>
       <c r="E4" t="n">
-        <v>22.3309425629695</v>
+        <v>22.33094256296949</v>
       </c>
       <c r="F4" t="n">
         <v>20.72818791946309</v>
       </c>
       <c r="G4" t="n">
-        <v>0.9282271834703389</v>
+        <v>0.9282271834703392</v>
       </c>
     </row>
     <row r="5">
@@ -8497,16 +8497,16 @@
         <v>20.72818791946309</v>
       </c>
       <c r="D5" t="n">
-        <v>22.3309425629695</v>
+        <v>22.33094256296949</v>
       </c>
       <c r="E5" t="n">
-        <v>22.3309425629695</v>
+        <v>22.33094256296949</v>
       </c>
       <c r="F5" t="n">
         <v>20.72818791946309</v>
       </c>
       <c r="G5" t="n">
-        <v>0.9282271834703389</v>
+        <v>0.9282271834703392</v>
       </c>
     </row>
     <row r="6">
@@ -9073,7 +9073,7 @@
         <v>128.7575503355705</v>
       </c>
       <c r="G26" t="n">
-        <v>6.056717079432987</v>
+        <v>6.056717079432986</v>
       </c>
     </row>
     <row r="27">
@@ -9100,7 +9100,7 @@
         <v>128.7575503355705</v>
       </c>
       <c r="G27" t="n">
-        <v>6.056717079432987</v>
+        <v>6.056717079432986</v>
       </c>
     </row>
     <row r="28">
@@ -9127,7 +9127,7 @@
         <v>128.7575503355705</v>
       </c>
       <c r="G28" t="n">
-        <v>6.056717079432987</v>
+        <v>6.056717079432986</v>
       </c>
     </row>
     <row r="29">
@@ -9154,7 +9154,7 @@
         <v>128.7575503355705</v>
       </c>
       <c r="G29" t="n">
-        <v>6.056717079432987</v>
+        <v>6.056717079432986</v>
       </c>
     </row>
     <row r="30">
@@ -9181,7 +9181,7 @@
         <v>128.7575503355705</v>
       </c>
       <c r="G30" t="n">
-        <v>6.056717079432987</v>
+        <v>6.056717079432986</v>
       </c>
     </row>
     <row r="31">
@@ -9208,7 +9208,7 @@
         <v>128.7575503355705</v>
       </c>
       <c r="G31" t="n">
-        <v>6.056717079432987</v>
+        <v>6.056717079432986</v>
       </c>
     </row>
     <row r="32">
@@ -9235,7 +9235,7 @@
         <v>128.7575503355705</v>
       </c>
       <c r="G32" t="n">
-        <v>6.056717079432987</v>
+        <v>6.056717079432986</v>
       </c>
     </row>
     <row r="33">
@@ -9262,7 +9262,7 @@
         <v>128.7575503355705</v>
       </c>
       <c r="G33" t="n">
-        <v>6.056717079432987</v>
+        <v>6.056717079432986</v>
       </c>
     </row>
     <row r="34">
@@ -9289,7 +9289,7 @@
         <v>128.7575503355705</v>
       </c>
       <c r="G34" t="n">
-        <v>6.056717079432987</v>
+        <v>6.056717079432986</v>
       </c>
     </row>
     <row r="35">
@@ -9316,7 +9316,7 @@
         <v>128.7575503355705</v>
       </c>
       <c r="G35" t="n">
-        <v>6.056717079432987</v>
+        <v>6.056717079432986</v>
       </c>
     </row>
     <row r="36">
@@ -9343,7 +9343,7 @@
         <v>128.7575503355705</v>
       </c>
       <c r="G36" t="n">
-        <v>6.056717079432987</v>
+        <v>6.056717079432986</v>
       </c>
     </row>
     <row r="37">
@@ -9370,7 +9370,7 @@
         <v>128.7575503355705</v>
       </c>
       <c r="G37" t="n">
-        <v>6.056717079432987</v>
+        <v>6.056717079432986</v>
       </c>
     </row>
     <row r="38">
@@ -9397,7 +9397,7 @@
         <v>128.7575503355705</v>
       </c>
       <c r="G38" t="n">
-        <v>6.056717079432987</v>
+        <v>6.056717079432986</v>
       </c>
     </row>
     <row r="39">
@@ -9424,7 +9424,7 @@
         <v>128.7575503355705</v>
       </c>
       <c r="G39" t="n">
-        <v>6.056717079432987</v>
+        <v>6.056717079432986</v>
       </c>
     </row>
     <row r="40">
@@ -9451,7 +9451,7 @@
         <v>128.7575503355705</v>
       </c>
       <c r="G40" t="n">
-        <v>6.056717079432987</v>
+        <v>6.056717079432986</v>
       </c>
     </row>
     <row r="41">
@@ -9478,7 +9478,7 @@
         <v>128.7575503355705</v>
       </c>
       <c r="G41" t="n">
-        <v>6.056717079432987</v>
+        <v>6.056717079432986</v>
       </c>
     </row>
     <row r="42">
@@ -9496,16 +9496,16 @@
         <v>20.72818791946309</v>
       </c>
       <c r="D42" t="n">
-        <v>22.3309425629695</v>
+        <v>22.33094256296949</v>
       </c>
       <c r="E42" t="n">
-        <v>22.3309425629695</v>
+        <v>22.33094256296949</v>
       </c>
       <c r="F42" t="n">
         <v>20.72818791946309</v>
       </c>
       <c r="G42" t="n">
-        <v>0.9282271834703389</v>
+        <v>0.9282271834703392</v>
       </c>
     </row>
     <row r="43">
@@ -9523,16 +9523,16 @@
         <v>20.72818791946309</v>
       </c>
       <c r="D43" t="n">
-        <v>22.3309425629695</v>
+        <v>22.33094256296949</v>
       </c>
       <c r="E43" t="n">
-        <v>22.3309425629695</v>
+        <v>22.33094256296949</v>
       </c>
       <c r="F43" t="n">
         <v>20.72818791946309</v>
       </c>
       <c r="G43" t="n">
-        <v>0.9282271834703389</v>
+        <v>0.9282271834703392</v>
       </c>
     </row>
     <row r="44">
@@ -9550,16 +9550,16 @@
         <v>20.72818791946309</v>
       </c>
       <c r="D44" t="n">
-        <v>22.3309425629695</v>
+        <v>22.33094256296949</v>
       </c>
       <c r="E44" t="n">
-        <v>22.3309425629695</v>
+        <v>22.33094256296949</v>
       </c>
       <c r="F44" t="n">
         <v>20.72818791946309</v>
       </c>
       <c r="G44" t="n">
-        <v>0.9282271834703389</v>
+        <v>0.9282271834703392</v>
       </c>
     </row>
     <row r="45">
@@ -9577,16 +9577,16 @@
         <v>20.72818791946309</v>
       </c>
       <c r="D45" t="n">
-        <v>22.3309425629695</v>
+        <v>22.33094256296949</v>
       </c>
       <c r="E45" t="n">
-        <v>22.3309425629695</v>
+        <v>22.33094256296949</v>
       </c>
       <c r="F45" t="n">
         <v>20.72818791946309</v>
       </c>
       <c r="G45" t="n">
-        <v>0.9282271834703389</v>
+        <v>0.9282271834703392</v>
       </c>
     </row>
     <row r="46">
@@ -9604,16 +9604,16 @@
         <v>20.72818791946309</v>
       </c>
       <c r="D46" t="n">
-        <v>22.3309425629695</v>
+        <v>22.33094256296949</v>
       </c>
       <c r="E46" t="n">
-        <v>22.3309425629695</v>
+        <v>22.33094256296949</v>
       </c>
       <c r="F46" t="n">
         <v>20.72818791946309</v>
       </c>
       <c r="G46" t="n">
-        <v>0.9282271834703389</v>
+        <v>0.9282271834703392</v>
       </c>
     </row>
     <row r="47">
@@ -9631,16 +9631,16 @@
         <v>20.72818791946309</v>
       </c>
       <c r="D47" t="n">
-        <v>22.3309425629695</v>
+        <v>22.33094256296949</v>
       </c>
       <c r="E47" t="n">
-        <v>22.3309425629695</v>
+        <v>22.33094256296949</v>
       </c>
       <c r="F47" t="n">
         <v>20.72818791946309</v>
       </c>
       <c r="G47" t="n">
-        <v>0.9282271834703389</v>
+        <v>0.9282271834703392</v>
       </c>
     </row>
     <row r="48">
@@ -9658,16 +9658,16 @@
         <v>20.72818791946309</v>
       </c>
       <c r="D48" t="n">
-        <v>22.3309425629695</v>
+        <v>22.33094256296949</v>
       </c>
       <c r="E48" t="n">
-        <v>22.3309425629695</v>
+        <v>22.33094256296949</v>
       </c>
       <c r="F48" t="n">
         <v>20.72818791946309</v>
       </c>
       <c r="G48" t="n">
-        <v>0.9282271834703389</v>
+        <v>0.9282271834703392</v>
       </c>
     </row>
     <row r="49">
@@ -9685,16 +9685,16 @@
         <v>20.72818791946309</v>
       </c>
       <c r="D49" t="n">
-        <v>22.3309425629695</v>
+        <v>22.33094256296949</v>
       </c>
       <c r="E49" t="n">
-        <v>22.3309425629695</v>
+        <v>22.33094256296949</v>
       </c>
       <c r="F49" t="n">
         <v>20.72818791946309</v>
       </c>
       <c r="G49" t="n">
-        <v>0.9282271834703389</v>
+        <v>0.9282271834703392</v>
       </c>
     </row>
     <row r="50">
@@ -9712,16 +9712,16 @@
         <v>20.72818791946309</v>
       </c>
       <c r="D50" t="n">
-        <v>22.3309425629695</v>
+        <v>22.33094256296949</v>
       </c>
       <c r="E50" t="n">
-        <v>22.3309425629695</v>
+        <v>22.33094256296949</v>
       </c>
       <c r="F50" t="n">
         <v>20.72818791946309</v>
       </c>
       <c r="G50" t="n">
-        <v>0.9282271834703389</v>
+        <v>0.9282271834703392</v>
       </c>
     </row>
     <row r="51">
@@ -9739,16 +9739,16 @@
         <v>20.72818791946309</v>
       </c>
       <c r="D51" t="n">
-        <v>22.3309425629695</v>
+        <v>22.33094256296949</v>
       </c>
       <c r="E51" t="n">
-        <v>22.3309425629695</v>
+        <v>22.33094256296949</v>
       </c>
       <c r="F51" t="n">
         <v>20.72818791946309</v>
       </c>
       <c r="G51" t="n">
-        <v>0.9282271834703389</v>
+        <v>0.9282271834703392</v>
       </c>
     </row>
     <row r="52">
@@ -9766,16 +9766,16 @@
         <v>20.72818791946309</v>
       </c>
       <c r="D52" t="n">
-        <v>22.3309425629695</v>
+        <v>22.33094256296949</v>
       </c>
       <c r="E52" t="n">
-        <v>22.3309425629695</v>
+        <v>22.33094256296949</v>
       </c>
       <c r="F52" t="n">
         <v>20.72818791946309</v>
       </c>
       <c r="G52" t="n">
-        <v>0.9282271834703389</v>
+        <v>0.9282271834703392</v>
       </c>
     </row>
     <row r="53">
@@ -9793,16 +9793,16 @@
         <v>20.72818791946309</v>
       </c>
       <c r="D53" t="n">
-        <v>22.3309425629695</v>
+        <v>22.33094256296949</v>
       </c>
       <c r="E53" t="n">
-        <v>22.3309425629695</v>
+        <v>22.33094256296949</v>
       </c>
       <c r="F53" t="n">
         <v>20.72818791946309</v>
       </c>
       <c r="G53" t="n">
-        <v>0.9282271834703389</v>
+        <v>0.9282271834703392</v>
       </c>
     </row>
     <row r="54">
@@ -9820,16 +9820,16 @@
         <v>20.72818791946309</v>
       </c>
       <c r="D54" t="n">
-        <v>22.3309425629695</v>
+        <v>22.33094256296949</v>
       </c>
       <c r="E54" t="n">
-        <v>22.3309425629695</v>
+        <v>22.33094256296949</v>
       </c>
       <c r="F54" t="n">
         <v>20.72818791946309</v>
       </c>
       <c r="G54" t="n">
-        <v>0.9282271834703389</v>
+        <v>0.9282271834703392</v>
       </c>
     </row>
     <row r="55">
@@ -9847,16 +9847,16 @@
         <v>20.72818791946309</v>
       </c>
       <c r="D55" t="n">
-        <v>22.3309425629695</v>
+        <v>22.33094256296949</v>
       </c>
       <c r="E55" t="n">
-        <v>22.3309425629695</v>
+        <v>22.33094256296949</v>
       </c>
       <c r="F55" t="n">
         <v>20.72818791946309</v>
       </c>
       <c r="G55" t="n">
-        <v>0.9282271834703389</v>
+        <v>0.9282271834703392</v>
       </c>
     </row>
     <row r="56">
@@ -9874,16 +9874,16 @@
         <v>20.72818791946309</v>
       </c>
       <c r="D56" t="n">
-        <v>22.3309425629695</v>
+        <v>22.33094256296949</v>
       </c>
       <c r="E56" t="n">
-        <v>22.3309425629695</v>
+        <v>22.33094256296949</v>
       </c>
       <c r="F56" t="n">
         <v>20.72818791946309</v>
       </c>
       <c r="G56" t="n">
-        <v>0.9282271834703389</v>
+        <v>0.9282271834703392</v>
       </c>
     </row>
     <row r="57">
@@ -9901,16 +9901,16 @@
         <v>20.72818791946309</v>
       </c>
       <c r="D57" t="n">
-        <v>22.3309425629695</v>
+        <v>22.33094256296949</v>
       </c>
       <c r="E57" t="n">
-        <v>22.3309425629695</v>
+        <v>22.33094256296949</v>
       </c>
       <c r="F57" t="n">
         <v>20.72818791946309</v>
       </c>
       <c r="G57" t="n">
-        <v>0.9282271834703389</v>
+        <v>0.9282271834703392</v>
       </c>
     </row>
     <row r="58">
@@ -9928,16 +9928,16 @@
         <v>20.72818791946309</v>
       </c>
       <c r="D58" t="n">
-        <v>22.3309425629695</v>
+        <v>22.33094256296949</v>
       </c>
       <c r="E58" t="n">
-        <v>22.3309425629695</v>
+        <v>22.33094256296949</v>
       </c>
       <c r="F58" t="n">
         <v>20.72818791946309</v>
       </c>
       <c r="G58" t="n">
-        <v>0.9282271834703389</v>
+        <v>0.9282271834703392</v>
       </c>
     </row>
     <row r="59">
@@ -9955,16 +9955,16 @@
         <v>20.72818791946309</v>
       </c>
       <c r="D59" t="n">
-        <v>22.3309425629695</v>
+        <v>22.33094256296949</v>
       </c>
       <c r="E59" t="n">
-        <v>22.3309425629695</v>
+        <v>22.33094256296949</v>
       </c>
       <c r="F59" t="n">
         <v>20.72818791946309</v>
       </c>
       <c r="G59" t="n">
-        <v>0.9282271834703389</v>
+        <v>0.9282271834703392</v>
       </c>
     </row>
     <row r="60">
@@ -9982,16 +9982,16 @@
         <v>20.72818791946309</v>
       </c>
       <c r="D60" t="n">
-        <v>22.3309425629695</v>
+        <v>22.33094256296949</v>
       </c>
       <c r="E60" t="n">
-        <v>22.3309425629695</v>
+        <v>22.33094256296949</v>
       </c>
       <c r="F60" t="n">
         <v>20.72818791946309</v>
       </c>
       <c r="G60" t="n">
-        <v>0.9282271834703389</v>
+        <v>0.9282271834703392</v>
       </c>
     </row>
     <row r="61">
@@ -10009,16 +10009,16 @@
         <v>20.72818791946309</v>
       </c>
       <c r="D61" t="n">
-        <v>22.3309425629695</v>
+        <v>22.33094256296949</v>
       </c>
       <c r="E61" t="n">
-        <v>22.3309425629695</v>
+        <v>22.33094256296949</v>
       </c>
       <c r="F61" t="n">
         <v>20.72818791946309</v>
       </c>
       <c r="G61" t="n">
-        <v>0.9282271834703389</v>
+        <v>0.9282271834703392</v>
       </c>
     </row>
     <row r="62">
@@ -10036,16 +10036,16 @@
         <v>20.72818791946309</v>
       </c>
       <c r="D62" t="n">
-        <v>22.3309425629695</v>
+        <v>22.33094256296949</v>
       </c>
       <c r="E62" t="n">
-        <v>22.3309425629695</v>
+        <v>22.33094256296949</v>
       </c>
       <c r="F62" t="n">
         <v>20.72818791946309</v>
       </c>
       <c r="G62" t="n">
-        <v>0.9282271834703389</v>
+        <v>0.9282271834703392</v>
       </c>
     </row>
     <row r="63">
@@ -10063,16 +10063,16 @@
         <v>20.72818791946309</v>
       </c>
       <c r="D63" t="n">
-        <v>22.3309425629695</v>
+        <v>22.33094256296949</v>
       </c>
       <c r="E63" t="n">
-        <v>22.3309425629695</v>
+        <v>22.33094256296949</v>
       </c>
       <c r="F63" t="n">
         <v>20.72818791946309</v>
       </c>
       <c r="G63" t="n">
-        <v>0.9282271834703389</v>
+        <v>0.9282271834703392</v>
       </c>
     </row>
     <row r="64">
@@ -10090,16 +10090,16 @@
         <v>20.72818791946309</v>
       </c>
       <c r="D64" t="n">
-        <v>22.3309425629695</v>
+        <v>22.33094256296949</v>
       </c>
       <c r="E64" t="n">
-        <v>22.3309425629695</v>
+        <v>22.33094256296949</v>
       </c>
       <c r="F64" t="n">
         <v>20.72818791946309</v>
       </c>
       <c r="G64" t="n">
-        <v>0.9282271834703389</v>
+        <v>0.9282271834703392</v>
       </c>
     </row>
     <row r="65">
@@ -10117,16 +10117,16 @@
         <v>20.72818791946309</v>
       </c>
       <c r="D65" t="n">
-        <v>22.3309425629695</v>
+        <v>22.33094256296949</v>
       </c>
       <c r="E65" t="n">
-        <v>22.3309425629695</v>
+        <v>22.33094256296949</v>
       </c>
       <c r="F65" t="n">
         <v>20.72818791946309</v>
       </c>
       <c r="G65" t="n">
-        <v>0.9282271834703389</v>
+        <v>0.9282271834703392</v>
       </c>
     </row>
     <row r="66">
@@ -10144,16 +10144,16 @@
         <v>20.72818791946309</v>
       </c>
       <c r="D66" t="n">
-        <v>22.3309425629695</v>
+        <v>22.33094256296949</v>
       </c>
       <c r="E66" t="n">
-        <v>22.3309425629695</v>
+        <v>22.33094256296949</v>
       </c>
       <c r="F66" t="n">
         <v>20.72818791946309</v>
       </c>
       <c r="G66" t="n">
-        <v>0.9282271834703389</v>
+        <v>0.9282271834703392</v>
       </c>
     </row>
     <row r="67">
@@ -10171,16 +10171,16 @@
         <v>20.72818791946309</v>
       </c>
       <c r="D67" t="n">
-        <v>22.3309425629695</v>
+        <v>22.33094256296949</v>
       </c>
       <c r="E67" t="n">
-        <v>22.3309425629695</v>
+        <v>22.33094256296949</v>
       </c>
       <c r="F67" t="n">
         <v>20.72818791946309</v>
       </c>
       <c r="G67" t="n">
-        <v>0.9282271834703389</v>
+        <v>0.9282271834703392</v>
       </c>
     </row>
     <row r="68">
@@ -10198,16 +10198,16 @@
         <v>20.72818791946309</v>
       </c>
       <c r="D68" t="n">
-        <v>22.3309425629695</v>
+        <v>22.33094256296949</v>
       </c>
       <c r="E68" t="n">
-        <v>22.3309425629695</v>
+        <v>22.33094256296949</v>
       </c>
       <c r="F68" t="n">
         <v>20.72818791946309</v>
       </c>
       <c r="G68" t="n">
-        <v>0.9282271834703389</v>
+        <v>0.9282271834703392</v>
       </c>
     </row>
     <row r="69">
@@ -10225,16 +10225,16 @@
         <v>20.72818791946309</v>
       </c>
       <c r="D69" t="n">
-        <v>22.3309425629695</v>
+        <v>22.33094256296949</v>
       </c>
       <c r="E69" t="n">
-        <v>22.3309425629695</v>
+        <v>22.33094256296949</v>
       </c>
       <c r="F69" t="n">
         <v>20.72818791946309</v>
       </c>
       <c r="G69" t="n">
-        <v>0.9282271834703389</v>
+        <v>0.9282271834703392</v>
       </c>
     </row>
     <row r="70">
@@ -14359,7 +14359,7 @@
         <v>383.95390625</v>
       </c>
       <c r="G26" t="n">
-        <v>14.39748662251902</v>
+        <v>14.39748662251903</v>
       </c>
     </row>
     <row r="27">
@@ -14386,7 +14386,7 @@
         <v>383.95390625</v>
       </c>
       <c r="G27" t="n">
-        <v>14.39748662251902</v>
+        <v>14.39748662251903</v>
       </c>
     </row>
     <row r="28">
@@ -14413,7 +14413,7 @@
         <v>383.95390625</v>
       </c>
       <c r="G28" t="n">
-        <v>14.39748662251902</v>
+        <v>14.39748662251903</v>
       </c>
     </row>
     <row r="29">
@@ -14440,7 +14440,7 @@
         <v>383.95390625</v>
       </c>
       <c r="G29" t="n">
-        <v>14.39748662251902</v>
+        <v>14.39748662251903</v>
       </c>
     </row>
     <row r="30">
@@ -14467,7 +14467,7 @@
         <v>383.95390625</v>
       </c>
       <c r="G30" t="n">
-        <v>14.39748662251902</v>
+        <v>14.39748662251903</v>
       </c>
     </row>
     <row r="31">
@@ -14494,7 +14494,7 @@
         <v>383.95390625</v>
       </c>
       <c r="G31" t="n">
-        <v>14.39748662251902</v>
+        <v>14.39748662251903</v>
       </c>
     </row>
     <row r="32">
@@ -14521,7 +14521,7 @@
         <v>383.95390625</v>
       </c>
       <c r="G32" t="n">
-        <v>14.39748662251902</v>
+        <v>14.39748662251903</v>
       </c>
     </row>
     <row r="33">
@@ -14548,7 +14548,7 @@
         <v>383.95390625</v>
       </c>
       <c r="G33" t="n">
-        <v>14.39748662251902</v>
+        <v>14.39748662251903</v>
       </c>
     </row>
     <row r="34">
@@ -14575,7 +14575,7 @@
         <v>383.95390625</v>
       </c>
       <c r="G34" t="n">
-        <v>14.39748662251902</v>
+        <v>14.39748662251903</v>
       </c>
     </row>
     <row r="35">
@@ -14602,7 +14602,7 @@
         <v>383.95390625</v>
       </c>
       <c r="G35" t="n">
-        <v>14.39748662251902</v>
+        <v>14.39748662251903</v>
       </c>
     </row>
     <row r="36">
@@ -14629,7 +14629,7 @@
         <v>383.95390625</v>
       </c>
       <c r="G36" t="n">
-        <v>14.39748662251902</v>
+        <v>14.39748662251903</v>
       </c>
     </row>
     <row r="37">
@@ -14656,7 +14656,7 @@
         <v>383.95390625</v>
       </c>
       <c r="G37" t="n">
-        <v>14.39748662251902</v>
+        <v>14.39748662251903</v>
       </c>
     </row>
     <row r="38">
@@ -14683,7 +14683,7 @@
         <v>383.95390625</v>
       </c>
       <c r="G38" t="n">
-        <v>14.39748662251902</v>
+        <v>14.39748662251903</v>
       </c>
     </row>
     <row r="39">
@@ -14710,7 +14710,7 @@
         <v>383.95390625</v>
       </c>
       <c r="G39" t="n">
-        <v>14.39748662251902</v>
+        <v>14.39748662251903</v>
       </c>
     </row>
     <row r="40">
@@ -14737,7 +14737,7 @@
         <v>383.95390625</v>
       </c>
       <c r="G40" t="n">
-        <v>14.39748662251902</v>
+        <v>14.39748662251903</v>
       </c>
     </row>
     <row r="41">
@@ -14764,7 +14764,7 @@
         <v>383.95390625</v>
       </c>
       <c r="G41" t="n">
-        <v>14.39748662251902</v>
+        <v>14.39748662251903</v>
       </c>
     </row>
     <row r="42">
@@ -15862,10 +15862,10 @@
         <v>343.06796875</v>
       </c>
       <c r="D82" t="n">
-        <v>27.25852457072115</v>
+        <v>27.25852457072116</v>
       </c>
       <c r="E82" t="n">
-        <v>27.25852457072115</v>
+        <v>27.25852457072116</v>
       </c>
       <c r="F82" t="n">
         <v>343.06796875</v>
@@ -15889,10 +15889,10 @@
         <v>343.06796875</v>
       </c>
       <c r="D83" t="n">
-        <v>27.25852457072115</v>
+        <v>27.25852457072116</v>
       </c>
       <c r="E83" t="n">
-        <v>27.25852457072115</v>
+        <v>27.25852457072116</v>
       </c>
       <c r="F83" t="n">
         <v>343.06796875</v>
@@ -15916,10 +15916,10 @@
         <v>343.06796875</v>
       </c>
       <c r="D84" t="n">
-        <v>27.25852457072115</v>
+        <v>27.25852457072116</v>
       </c>
       <c r="E84" t="n">
-        <v>27.25852457072115</v>
+        <v>27.25852457072116</v>
       </c>
       <c r="F84" t="n">
         <v>343.06796875</v>
@@ -15943,10 +15943,10 @@
         <v>343.06796875</v>
       </c>
       <c r="D85" t="n">
-        <v>27.25852457072115</v>
+        <v>27.25852457072116</v>
       </c>
       <c r="E85" t="n">
-        <v>27.25852457072115</v>
+        <v>27.25852457072116</v>
       </c>
       <c r="F85" t="n">
         <v>343.06796875</v>
@@ -15970,10 +15970,10 @@
         <v>343.06796875</v>
       </c>
       <c r="D86" t="n">
-        <v>27.25852457072115</v>
+        <v>27.25852457072116</v>
       </c>
       <c r="E86" t="n">
-        <v>27.25852457072115</v>
+        <v>27.25852457072116</v>
       </c>
       <c r="F86" t="n">
         <v>343.06796875</v>
@@ -15997,10 +15997,10 @@
         <v>343.06796875</v>
       </c>
       <c r="D87" t="n">
-        <v>27.25852457072115</v>
+        <v>27.25852457072116</v>
       </c>
       <c r="E87" t="n">
-        <v>27.25852457072115</v>
+        <v>27.25852457072116</v>
       </c>
       <c r="F87" t="n">
         <v>343.06796875</v>
@@ -16024,10 +16024,10 @@
         <v>343.06796875</v>
       </c>
       <c r="D88" t="n">
-        <v>27.25852457072115</v>
+        <v>27.25852457072116</v>
       </c>
       <c r="E88" t="n">
-        <v>27.25852457072115</v>
+        <v>27.25852457072116</v>
       </c>
       <c r="F88" t="n">
         <v>343.06796875</v>
@@ -16051,10 +16051,10 @@
         <v>343.06796875</v>
       </c>
       <c r="D89" t="n">
-        <v>27.25852457072115</v>
+        <v>27.25852457072116</v>
       </c>
       <c r="E89" t="n">
-        <v>27.25852457072115</v>
+        <v>27.25852457072116</v>
       </c>
       <c r="F89" t="n">
         <v>343.06796875</v>
@@ -16078,10 +16078,10 @@
         <v>343.06796875</v>
       </c>
       <c r="D90" t="n">
-        <v>27.25852457072115</v>
+        <v>27.25852457072116</v>
       </c>
       <c r="E90" t="n">
-        <v>27.25852457072115</v>
+        <v>27.25852457072116</v>
       </c>
       <c r="F90" t="n">
         <v>343.06796875</v>
@@ -16105,10 +16105,10 @@
         <v>343.06796875</v>
       </c>
       <c r="D91" t="n">
-        <v>27.25852457072115</v>
+        <v>27.25852457072116</v>
       </c>
       <c r="E91" t="n">
-        <v>27.25852457072115</v>
+        <v>27.25852457072116</v>
       </c>
       <c r="F91" t="n">
         <v>343.06796875</v>
@@ -16132,10 +16132,10 @@
         <v>343.06796875</v>
       </c>
       <c r="D92" t="n">
-        <v>27.25852457072115</v>
+        <v>27.25852457072116</v>
       </c>
       <c r="E92" t="n">
-        <v>27.25852457072115</v>
+        <v>27.25852457072116</v>
       </c>
       <c r="F92" t="n">
         <v>343.06796875</v>
@@ -16159,10 +16159,10 @@
         <v>343.06796875</v>
       </c>
       <c r="D93" t="n">
-        <v>27.25852457072115</v>
+        <v>27.25852457072116</v>
       </c>
       <c r="E93" t="n">
-        <v>27.25852457072115</v>
+        <v>27.25852457072116</v>
       </c>
       <c r="F93" t="n">
         <v>343.06796875</v>
@@ -16186,10 +16186,10 @@
         <v>343.06796875</v>
       </c>
       <c r="D94" t="n">
-        <v>27.25852457072115</v>
+        <v>27.25852457072116</v>
       </c>
       <c r="E94" t="n">
-        <v>27.25852457072115</v>
+        <v>27.25852457072116</v>
       </c>
       <c r="F94" t="n">
         <v>343.06796875</v>
@@ -16213,10 +16213,10 @@
         <v>343.06796875</v>
       </c>
       <c r="D95" t="n">
-        <v>27.25852457072115</v>
+        <v>27.25852457072116</v>
       </c>
       <c r="E95" t="n">
-        <v>27.25852457072115</v>
+        <v>27.25852457072116</v>
       </c>
       <c r="F95" t="n">
         <v>343.06796875</v>
@@ -16240,10 +16240,10 @@
         <v>343.06796875</v>
       </c>
       <c r="D96" t="n">
-        <v>27.25852457072115</v>
+        <v>27.25852457072116</v>
       </c>
       <c r="E96" t="n">
-        <v>27.25852457072115</v>
+        <v>27.25852457072116</v>
       </c>
       <c r="F96" t="n">
         <v>343.06796875</v>
@@ -16267,10 +16267,10 @@
         <v>343.06796875</v>
       </c>
       <c r="D97" t="n">
-        <v>27.25852457072115</v>
+        <v>27.25852457072116</v>
       </c>
       <c r="E97" t="n">
-        <v>27.25852457072115</v>
+        <v>27.25852457072116</v>
       </c>
       <c r="F97" t="n">
         <v>343.06796875</v>
@@ -23788,7 +23788,7 @@
         </is>
       </c>
       <c r="C82" t="n">
-        <v>249.5268096514746</v>
+        <v>249.5268096514745</v>
       </c>
       <c r="D82" t="n">
         <v>26.98745470049381</v>
@@ -23797,10 +23797,10 @@
         <v>26.98745470049381</v>
       </c>
       <c r="F82" t="n">
-        <v>249.5268096514746</v>
+        <v>249.5268096514745</v>
       </c>
       <c r="G82" t="n">
-        <v>9.246029772748772</v>
+        <v>9.24602977274877</v>
       </c>
     </row>
     <row r="83">
@@ -23815,7 +23815,7 @@
         </is>
       </c>
       <c r="C83" t="n">
-        <v>249.5268096514746</v>
+        <v>249.5268096514745</v>
       </c>
       <c r="D83" t="n">
         <v>26.98745470049381</v>
@@ -23824,10 +23824,10 @@
         <v>26.98745470049381</v>
       </c>
       <c r="F83" t="n">
-        <v>249.5268096514746</v>
+        <v>249.5268096514745</v>
       </c>
       <c r="G83" t="n">
-        <v>9.246029772748772</v>
+        <v>9.24602977274877</v>
       </c>
     </row>
     <row r="84">
@@ -23842,7 +23842,7 @@
         </is>
       </c>
       <c r="C84" t="n">
-        <v>249.5268096514746</v>
+        <v>249.5268096514745</v>
       </c>
       <c r="D84" t="n">
         <v>26.98745470049381</v>
@@ -23851,10 +23851,10 @@
         <v>26.98745470049381</v>
       </c>
       <c r="F84" t="n">
-        <v>249.5268096514746</v>
+        <v>249.5268096514745</v>
       </c>
       <c r="G84" t="n">
-        <v>9.246029772748772</v>
+        <v>9.24602977274877</v>
       </c>
     </row>
     <row r="85">
@@ -23869,7 +23869,7 @@
         </is>
       </c>
       <c r="C85" t="n">
-        <v>249.5268096514746</v>
+        <v>249.5268096514745</v>
       </c>
       <c r="D85" t="n">
         <v>26.98745470049381</v>
@@ -23878,10 +23878,10 @@
         <v>26.98745470049381</v>
       </c>
       <c r="F85" t="n">
-        <v>249.5268096514746</v>
+        <v>249.5268096514745</v>
       </c>
       <c r="G85" t="n">
-        <v>9.246029772748772</v>
+        <v>9.24602977274877</v>
       </c>
     </row>
     <row r="86">
@@ -23896,7 +23896,7 @@
         </is>
       </c>
       <c r="C86" t="n">
-        <v>249.5268096514746</v>
+        <v>249.5268096514745</v>
       </c>
       <c r="D86" t="n">
         <v>26.98745470049381</v>
@@ -23905,10 +23905,10 @@
         <v>26.98745470049381</v>
       </c>
       <c r="F86" t="n">
-        <v>249.5268096514746</v>
+        <v>249.5268096514745</v>
       </c>
       <c r="G86" t="n">
-        <v>9.246029772748772</v>
+        <v>9.24602977274877</v>
       </c>
     </row>
     <row r="87">
@@ -23923,7 +23923,7 @@
         </is>
       </c>
       <c r="C87" t="n">
-        <v>249.5268096514746</v>
+        <v>249.5268096514745</v>
       </c>
       <c r="D87" t="n">
         <v>26.98745470049381</v>
@@ -23932,10 +23932,10 @@
         <v>26.98745470049381</v>
       </c>
       <c r="F87" t="n">
-        <v>249.5268096514746</v>
+        <v>249.5268096514745</v>
       </c>
       <c r="G87" t="n">
-        <v>9.246029772748772</v>
+        <v>9.24602977274877</v>
       </c>
     </row>
     <row r="88">
@@ -23950,7 +23950,7 @@
         </is>
       </c>
       <c r="C88" t="n">
-        <v>249.5268096514746</v>
+        <v>249.5268096514745</v>
       </c>
       <c r="D88" t="n">
         <v>26.98745470049381</v>
@@ -23959,10 +23959,10 @@
         <v>26.98745470049381</v>
       </c>
       <c r="F88" t="n">
-        <v>249.5268096514746</v>
+        <v>249.5268096514745</v>
       </c>
       <c r="G88" t="n">
-        <v>9.246029772748772</v>
+        <v>9.24602977274877</v>
       </c>
     </row>
     <row r="89">
@@ -23977,7 +23977,7 @@
         </is>
       </c>
       <c r="C89" t="n">
-        <v>249.5268096514746</v>
+        <v>249.5268096514745</v>
       </c>
       <c r="D89" t="n">
         <v>26.98745470049381</v>
@@ -23986,10 +23986,10 @@
         <v>26.98745470049381</v>
       </c>
       <c r="F89" t="n">
-        <v>249.5268096514746</v>
+        <v>249.5268096514745</v>
       </c>
       <c r="G89" t="n">
-        <v>9.246029772748772</v>
+        <v>9.24602977274877</v>
       </c>
     </row>
     <row r="90">
@@ -24004,7 +24004,7 @@
         </is>
       </c>
       <c r="C90" t="n">
-        <v>249.5268096514746</v>
+        <v>249.5268096514745</v>
       </c>
       <c r="D90" t="n">
         <v>26.98745470049381</v>
@@ -24013,10 +24013,10 @@
         <v>26.98745470049381</v>
       </c>
       <c r="F90" t="n">
-        <v>249.5268096514746</v>
+        <v>249.5268096514745</v>
       </c>
       <c r="G90" t="n">
-        <v>9.246029772748772</v>
+        <v>9.24602977274877</v>
       </c>
     </row>
     <row r="91">
@@ -24031,7 +24031,7 @@
         </is>
       </c>
       <c r="C91" t="n">
-        <v>249.5268096514746</v>
+        <v>249.5268096514745</v>
       </c>
       <c r="D91" t="n">
         <v>26.98745470049381</v>
@@ -24040,10 +24040,10 @@
         <v>26.98745470049381</v>
       </c>
       <c r="F91" t="n">
-        <v>249.5268096514746</v>
+        <v>249.5268096514745</v>
       </c>
       <c r="G91" t="n">
-        <v>9.246029772748772</v>
+        <v>9.24602977274877</v>
       </c>
     </row>
     <row r="92">
@@ -24058,7 +24058,7 @@
         </is>
       </c>
       <c r="C92" t="n">
-        <v>249.5268096514746</v>
+        <v>249.5268096514745</v>
       </c>
       <c r="D92" t="n">
         <v>26.98745470049381</v>
@@ -24067,10 +24067,10 @@
         <v>26.98745470049381</v>
       </c>
       <c r="F92" t="n">
-        <v>249.5268096514746</v>
+        <v>249.5268096514745</v>
       </c>
       <c r="G92" t="n">
-        <v>9.246029772748772</v>
+        <v>9.24602977274877</v>
       </c>
     </row>
     <row r="93">
@@ -24085,7 +24085,7 @@
         </is>
       </c>
       <c r="C93" t="n">
-        <v>249.5268096514746</v>
+        <v>249.5268096514745</v>
       </c>
       <c r="D93" t="n">
         <v>26.98745470049381</v>
@@ -24094,10 +24094,10 @@
         <v>26.98745470049381</v>
       </c>
       <c r="F93" t="n">
-        <v>249.5268096514746</v>
+        <v>249.5268096514745</v>
       </c>
       <c r="G93" t="n">
-        <v>9.246029772748772</v>
+        <v>9.24602977274877</v>
       </c>
     </row>
     <row r="94">
@@ -24112,7 +24112,7 @@
         </is>
       </c>
       <c r="C94" t="n">
-        <v>249.5268096514746</v>
+        <v>249.5268096514745</v>
       </c>
       <c r="D94" t="n">
         <v>26.98745470049381</v>
@@ -24121,10 +24121,10 @@
         <v>26.98745470049381</v>
       </c>
       <c r="F94" t="n">
-        <v>249.5268096514746</v>
+        <v>249.5268096514745</v>
       </c>
       <c r="G94" t="n">
-        <v>9.246029772748772</v>
+        <v>9.24602977274877</v>
       </c>
     </row>
     <row r="95">
@@ -24139,7 +24139,7 @@
         </is>
       </c>
       <c r="C95" t="n">
-        <v>249.5268096514746</v>
+        <v>249.5268096514745</v>
       </c>
       <c r="D95" t="n">
         <v>26.98745470049381</v>
@@ -24148,10 +24148,10 @@
         <v>26.98745470049381</v>
       </c>
       <c r="F95" t="n">
-        <v>249.5268096514746</v>
+        <v>249.5268096514745</v>
       </c>
       <c r="G95" t="n">
-        <v>9.246029772748772</v>
+        <v>9.24602977274877</v>
       </c>
     </row>
     <row r="96">
@@ -24166,7 +24166,7 @@
         </is>
       </c>
       <c r="C96" t="n">
-        <v>249.5268096514746</v>
+        <v>249.5268096514745</v>
       </c>
       <c r="D96" t="n">
         <v>26.98745470049381</v>
@@ -24175,10 +24175,10 @@
         <v>26.98745470049381</v>
       </c>
       <c r="F96" t="n">
-        <v>249.5268096514746</v>
+        <v>249.5268096514745</v>
       </c>
       <c r="G96" t="n">
-        <v>9.246029772748772</v>
+        <v>9.24602977274877</v>
       </c>
     </row>
     <row r="97">
@@ -24193,7 +24193,7 @@
         </is>
       </c>
       <c r="C97" t="n">
-        <v>249.5268096514746</v>
+        <v>249.5268096514745</v>
       </c>
       <c r="D97" t="n">
         <v>26.98745470049381</v>
@@ -24202,10 +24202,10 @@
         <v>26.98745470049381</v>
       </c>
       <c r="F97" t="n">
-        <v>249.5268096514746</v>
+        <v>249.5268096514745</v>
       </c>
       <c r="G97" t="n">
-        <v>9.246029772748772</v>
+        <v>9.24602977274877</v>
       </c>
     </row>
   </sheetData>
@@ -34963,7 +34963,7 @@
         <v>270.9524752475248</v>
       </c>
       <c r="G6" t="n">
-        <v>14.31036423844835</v>
+        <v>14.31036423844836</v>
       </c>
     </row>
     <row r="7">
@@ -34990,7 +34990,7 @@
         <v>270.9524752475248</v>
       </c>
       <c r="G7" t="n">
-        <v>14.31036423844835</v>
+        <v>14.31036423844836</v>
       </c>
     </row>
     <row r="8">
@@ -35017,7 +35017,7 @@
         <v>270.9524752475248</v>
       </c>
       <c r="G8" t="n">
-        <v>14.31036423844835</v>
+        <v>14.31036423844836</v>
       </c>
     </row>
     <row r="9">
@@ -35044,7 +35044,7 @@
         <v>270.9524752475248</v>
       </c>
       <c r="G9" t="n">
-        <v>14.31036423844835</v>
+        <v>14.31036423844836</v>
       </c>
     </row>
     <row r="10">
@@ -35071,7 +35071,7 @@
         <v>270.9524752475248</v>
       </c>
       <c r="G10" t="n">
-        <v>14.31036423844835</v>
+        <v>14.31036423844836</v>
       </c>
     </row>
     <row r="11">
@@ -35098,7 +35098,7 @@
         <v>270.9524752475248</v>
       </c>
       <c r="G11" t="n">
-        <v>14.31036423844835</v>
+        <v>14.31036423844836</v>
       </c>
     </row>
     <row r="12">
@@ -35125,7 +35125,7 @@
         <v>270.9524752475248</v>
       </c>
       <c r="G12" t="n">
-        <v>14.31036423844835</v>
+        <v>14.31036423844836</v>
       </c>
     </row>
     <row r="13">
@@ -35152,7 +35152,7 @@
         <v>270.9524752475248</v>
       </c>
       <c r="G13" t="n">
-        <v>14.31036423844835</v>
+        <v>14.31036423844836</v>
       </c>
     </row>
     <row r="14">
@@ -35179,7 +35179,7 @@
         <v>270.9524752475248</v>
       </c>
       <c r="G14" t="n">
-        <v>14.31036423844835</v>
+        <v>14.31036423844836</v>
       </c>
     </row>
     <row r="15">
@@ -35206,7 +35206,7 @@
         <v>270.9524752475248</v>
       </c>
       <c r="G15" t="n">
-        <v>14.31036423844835</v>
+        <v>14.31036423844836</v>
       </c>
     </row>
     <row r="16">
@@ -35233,7 +35233,7 @@
         <v>270.9524752475248</v>
       </c>
       <c r="G16" t="n">
-        <v>14.31036423844835</v>
+        <v>14.31036423844836</v>
       </c>
     </row>
     <row r="17">
@@ -35260,7 +35260,7 @@
         <v>270.9524752475248</v>
       </c>
       <c r="G17" t="n">
-        <v>14.31036423844835</v>
+        <v>14.31036423844836</v>
       </c>
     </row>
     <row r="18">
@@ -35287,7 +35287,7 @@
         <v>270.9524752475248</v>
       </c>
       <c r="G18" t="n">
-        <v>14.31036423844835</v>
+        <v>14.31036423844836</v>
       </c>
     </row>
     <row r="19">
@@ -35314,7 +35314,7 @@
         <v>270.9524752475248</v>
       </c>
       <c r="G19" t="n">
-        <v>14.31036423844835</v>
+        <v>14.31036423844836</v>
       </c>
     </row>
     <row r="20">
@@ -35341,7 +35341,7 @@
         <v>270.9524752475248</v>
       </c>
       <c r="G20" t="n">
-        <v>14.31036423844835</v>
+        <v>14.31036423844836</v>
       </c>
     </row>
     <row r="21">
@@ -35368,7 +35368,7 @@
         <v>270.9524752475248</v>
       </c>
       <c r="G21" t="n">
-        <v>14.31036423844835</v>
+        <v>14.31036423844836</v>
       </c>
     </row>
     <row r="22">
@@ -35395,7 +35395,7 @@
         <v>270.9524752475248</v>
       </c>
       <c r="G22" t="n">
-        <v>14.31036423844835</v>
+        <v>14.31036423844836</v>
       </c>
     </row>
     <row r="23">
@@ -35422,7 +35422,7 @@
         <v>270.9524752475248</v>
       </c>
       <c r="G23" t="n">
-        <v>14.31036423844835</v>
+        <v>14.31036423844836</v>
       </c>
     </row>
     <row r="24">
@@ -35449,7 +35449,7 @@
         <v>270.9524752475248</v>
       </c>
       <c r="G24" t="n">
-        <v>14.31036423844835</v>
+        <v>14.31036423844836</v>
       </c>
     </row>
     <row r="25">
@@ -35476,7 +35476,7 @@
         <v>270.9524752475248</v>
       </c>
       <c r="G25" t="n">
-        <v>14.31036423844835</v>
+        <v>14.31036423844836</v>
       </c>
     </row>
     <row r="26">
@@ -36682,10 +36682,10 @@
         <v>22.01485148514852</v>
       </c>
       <c r="D70" t="n">
-        <v>20.53251868023359</v>
+        <v>20.5325186802336</v>
       </c>
       <c r="E70" t="n">
-        <v>20.53251868023359</v>
+        <v>20.5325186802336</v>
       </c>
       <c r="F70" t="n">
         <v>22.01485148514852</v>
@@ -36709,10 +36709,10 @@
         <v>22.01485148514852</v>
       </c>
       <c r="D71" t="n">
-        <v>20.53251868023359</v>
+        <v>20.5325186802336</v>
       </c>
       <c r="E71" t="n">
-        <v>20.53251868023359</v>
+        <v>20.5325186802336</v>
       </c>
       <c r="F71" t="n">
         <v>22.01485148514852</v>
@@ -36736,10 +36736,10 @@
         <v>22.01485148514852</v>
       </c>
       <c r="D72" t="n">
-        <v>20.53251868023359</v>
+        <v>20.5325186802336</v>
       </c>
       <c r="E72" t="n">
-        <v>20.53251868023359</v>
+        <v>20.5325186802336</v>
       </c>
       <c r="F72" t="n">
         <v>22.01485148514852</v>
@@ -36763,10 +36763,10 @@
         <v>22.01485148514852</v>
       </c>
       <c r="D73" t="n">
-        <v>20.53251868023359</v>
+        <v>20.5325186802336</v>
       </c>
       <c r="E73" t="n">
-        <v>20.53251868023359</v>
+        <v>20.5325186802336</v>
       </c>
       <c r="F73" t="n">
         <v>22.01485148514852</v>
@@ -36790,10 +36790,10 @@
         <v>22.01485148514852</v>
       </c>
       <c r="D74" t="n">
-        <v>20.53251868023359</v>
+        <v>20.5325186802336</v>
       </c>
       <c r="E74" t="n">
-        <v>20.53251868023359</v>
+        <v>20.5325186802336</v>
       </c>
       <c r="F74" t="n">
         <v>22.01485148514852</v>
@@ -36817,10 +36817,10 @@
         <v>22.01485148514852</v>
       </c>
       <c r="D75" t="n">
-        <v>20.53251868023359</v>
+        <v>20.5325186802336</v>
       </c>
       <c r="E75" t="n">
-        <v>20.53251868023359</v>
+        <v>20.5325186802336</v>
       </c>
       <c r="F75" t="n">
         <v>22.01485148514852</v>
@@ -36844,10 +36844,10 @@
         <v>22.01485148514852</v>
       </c>
       <c r="D76" t="n">
-        <v>20.53251868023359</v>
+        <v>20.5325186802336</v>
       </c>
       <c r="E76" t="n">
-        <v>20.53251868023359</v>
+        <v>20.5325186802336</v>
       </c>
       <c r="F76" t="n">
         <v>22.01485148514852</v>
@@ -36871,10 +36871,10 @@
         <v>22.01485148514852</v>
       </c>
       <c r="D77" t="n">
-        <v>20.53251868023359</v>
+        <v>20.5325186802336</v>
       </c>
       <c r="E77" t="n">
-        <v>20.53251868023359</v>
+        <v>20.5325186802336</v>
       </c>
       <c r="F77" t="n">
         <v>22.01485148514852</v>
@@ -36898,10 +36898,10 @@
         <v>22.01485148514852</v>
       </c>
       <c r="D78" t="n">
-        <v>20.53251868023359</v>
+        <v>20.5325186802336</v>
       </c>
       <c r="E78" t="n">
-        <v>20.53251868023359</v>
+        <v>20.5325186802336</v>
       </c>
       <c r="F78" t="n">
         <v>22.01485148514852</v>
@@ -36925,10 +36925,10 @@
         <v>22.01485148514852</v>
       </c>
       <c r="D79" t="n">
-        <v>20.53251868023359</v>
+        <v>20.5325186802336</v>
       </c>
       <c r="E79" t="n">
-        <v>20.53251868023359</v>
+        <v>20.5325186802336</v>
       </c>
       <c r="F79" t="n">
         <v>22.01485148514852</v>
@@ -36952,10 +36952,10 @@
         <v>22.01485148514852</v>
       </c>
       <c r="D80" t="n">
-        <v>20.53251868023359</v>
+        <v>20.5325186802336</v>
       </c>
       <c r="E80" t="n">
-        <v>20.53251868023359</v>
+        <v>20.5325186802336</v>
       </c>
       <c r="F80" t="n">
         <v>22.01485148514852</v>
@@ -36979,10 +36979,10 @@
         <v>22.01485148514852</v>
       </c>
       <c r="D81" t="n">
-        <v>20.53251868023359</v>
+        <v>20.5325186802336</v>
       </c>
       <c r="E81" t="n">
-        <v>20.53251868023359</v>
+        <v>20.5325186802336</v>
       </c>
       <c r="F81" t="n">
         <v>22.01485148514852</v>
@@ -37606,7 +37606,7 @@
         <v>268.8449122807017</v>
       </c>
       <c r="G6" t="n">
-        <v>15.04535199936728</v>
+        <v>15.04535199936727</v>
       </c>
     </row>
     <row r="7">
@@ -37633,7 +37633,7 @@
         <v>268.8449122807017</v>
       </c>
       <c r="G7" t="n">
-        <v>15.04535199936728</v>
+        <v>15.04535199936727</v>
       </c>
     </row>
     <row r="8">
@@ -37660,7 +37660,7 @@
         <v>268.8449122807017</v>
       </c>
       <c r="G8" t="n">
-        <v>15.04535199936728</v>
+        <v>15.04535199936727</v>
       </c>
     </row>
     <row r="9">
@@ -37687,7 +37687,7 @@
         <v>268.8449122807017</v>
       </c>
       <c r="G9" t="n">
-        <v>15.04535199936728</v>
+        <v>15.04535199936727</v>
       </c>
     </row>
     <row r="10">
@@ -37714,7 +37714,7 @@
         <v>268.8449122807017</v>
       </c>
       <c r="G10" t="n">
-        <v>15.04535199936728</v>
+        <v>15.04535199936727</v>
       </c>
     </row>
     <row r="11">
@@ -37741,7 +37741,7 @@
         <v>268.8449122807017</v>
       </c>
       <c r="G11" t="n">
-        <v>15.04535199936728</v>
+        <v>15.04535199936727</v>
       </c>
     </row>
     <row r="12">
@@ -37768,7 +37768,7 @@
         <v>268.8449122807017</v>
       </c>
       <c r="G12" t="n">
-        <v>15.04535199936728</v>
+        <v>15.04535199936727</v>
       </c>
     </row>
     <row r="13">
@@ -37795,7 +37795,7 @@
         <v>268.8449122807017</v>
       </c>
       <c r="G13" t="n">
-        <v>15.04535199936728</v>
+        <v>15.04535199936727</v>
       </c>
     </row>
     <row r="14">
@@ -37822,7 +37822,7 @@
         <v>268.8449122807017</v>
       </c>
       <c r="G14" t="n">
-        <v>15.04535199936728</v>
+        <v>15.04535199936727</v>
       </c>
     </row>
     <row r="15">
@@ -37849,7 +37849,7 @@
         <v>268.8449122807017</v>
       </c>
       <c r="G15" t="n">
-        <v>15.04535199936728</v>
+        <v>15.04535199936727</v>
       </c>
     </row>
     <row r="16">
@@ -37876,7 +37876,7 @@
         <v>268.8449122807017</v>
       </c>
       <c r="G16" t="n">
-        <v>15.04535199936728</v>
+        <v>15.04535199936727</v>
       </c>
     </row>
     <row r="17">
@@ -37903,7 +37903,7 @@
         <v>268.8449122807017</v>
       </c>
       <c r="G17" t="n">
-        <v>15.04535199936728</v>
+        <v>15.04535199936727</v>
       </c>
     </row>
     <row r="18">
@@ -37930,7 +37930,7 @@
         <v>268.8449122807017</v>
       </c>
       <c r="G18" t="n">
-        <v>15.04535199936728</v>
+        <v>15.04535199936727</v>
       </c>
     </row>
     <row r="19">
@@ -37957,7 +37957,7 @@
         <v>268.8449122807017</v>
       </c>
       <c r="G19" t="n">
-        <v>15.04535199936728</v>
+        <v>15.04535199936727</v>
       </c>
     </row>
     <row r="20">
@@ -37984,7 +37984,7 @@
         <v>268.8449122807017</v>
       </c>
       <c r="G20" t="n">
-        <v>15.04535199936728</v>
+        <v>15.04535199936727</v>
       </c>
     </row>
     <row r="21">
@@ -38011,7 +38011,7 @@
         <v>268.8449122807017</v>
       </c>
       <c r="G21" t="n">
-        <v>15.04535199936728</v>
+        <v>15.04535199936727</v>
       </c>
     </row>
     <row r="22">
@@ -38038,7 +38038,7 @@
         <v>268.8449122807017</v>
       </c>
       <c r="G22" t="n">
-        <v>15.04535199936728</v>
+        <v>15.04535199936727</v>
       </c>
     </row>
     <row r="23">
@@ -38065,7 +38065,7 @@
         <v>268.8449122807017</v>
       </c>
       <c r="G23" t="n">
-        <v>15.04535199936728</v>
+        <v>15.04535199936727</v>
       </c>
     </row>
     <row r="24">
@@ -38092,7 +38092,7 @@
         <v>268.8449122807017</v>
       </c>
       <c r="G24" t="n">
-        <v>15.04535199936728</v>
+        <v>15.04535199936727</v>
       </c>
     </row>
     <row r="25">
@@ -38119,7 +38119,7 @@
         <v>268.8449122807017</v>
       </c>
       <c r="G25" t="n">
-        <v>15.04535199936728</v>
+        <v>15.04535199936727</v>
       </c>
     </row>
     <row r="26">
@@ -39325,10 +39325,10 @@
         <v>25.65964912280701</v>
       </c>
       <c r="D70" t="n">
-        <v>19.62430811506723</v>
+        <v>19.62430811506724</v>
       </c>
       <c r="E70" t="n">
-        <v>19.62430811506723</v>
+        <v>19.62430811506724</v>
       </c>
       <c r="F70" t="n">
         <v>25.65964912280701</v>
@@ -39352,10 +39352,10 @@
         <v>25.65964912280701</v>
       </c>
       <c r="D71" t="n">
-        <v>19.62430811506723</v>
+        <v>19.62430811506724</v>
       </c>
       <c r="E71" t="n">
-        <v>19.62430811506723</v>
+        <v>19.62430811506724</v>
       </c>
       <c r="F71" t="n">
         <v>25.65964912280701</v>
@@ -39379,10 +39379,10 @@
         <v>25.65964912280701</v>
       </c>
       <c r="D72" t="n">
-        <v>19.62430811506723</v>
+        <v>19.62430811506724</v>
       </c>
       <c r="E72" t="n">
-        <v>19.62430811506723</v>
+        <v>19.62430811506724</v>
       </c>
       <c r="F72" t="n">
         <v>25.65964912280701</v>
@@ -39406,10 +39406,10 @@
         <v>25.65964912280701</v>
       </c>
       <c r="D73" t="n">
-        <v>19.62430811506723</v>
+        <v>19.62430811506724</v>
       </c>
       <c r="E73" t="n">
-        <v>19.62430811506723</v>
+        <v>19.62430811506724</v>
       </c>
       <c r="F73" t="n">
         <v>25.65964912280701</v>
@@ -39433,10 +39433,10 @@
         <v>25.65964912280701</v>
       </c>
       <c r="D74" t="n">
-        <v>19.62430811506723</v>
+        <v>19.62430811506724</v>
       </c>
       <c r="E74" t="n">
-        <v>19.62430811506723</v>
+        <v>19.62430811506724</v>
       </c>
       <c r="F74" t="n">
         <v>25.65964912280701</v>
@@ -39460,10 +39460,10 @@
         <v>25.65964912280701</v>
       </c>
       <c r="D75" t="n">
-        <v>19.62430811506723</v>
+        <v>19.62430811506724</v>
       </c>
       <c r="E75" t="n">
-        <v>19.62430811506723</v>
+        <v>19.62430811506724</v>
       </c>
       <c r="F75" t="n">
         <v>25.65964912280701</v>
@@ -39487,10 +39487,10 @@
         <v>25.65964912280701</v>
       </c>
       <c r="D76" t="n">
-        <v>19.62430811506723</v>
+        <v>19.62430811506724</v>
       </c>
       <c r="E76" t="n">
-        <v>19.62430811506723</v>
+        <v>19.62430811506724</v>
       </c>
       <c r="F76" t="n">
         <v>25.65964912280701</v>
@@ -39514,10 +39514,10 @@
         <v>25.65964912280701</v>
       </c>
       <c r="D77" t="n">
-        <v>19.62430811506723</v>
+        <v>19.62430811506724</v>
       </c>
       <c r="E77" t="n">
-        <v>19.62430811506723</v>
+        <v>19.62430811506724</v>
       </c>
       <c r="F77" t="n">
         <v>25.65964912280701</v>
@@ -39541,10 +39541,10 @@
         <v>25.65964912280701</v>
       </c>
       <c r="D78" t="n">
-        <v>19.62430811506723</v>
+        <v>19.62430811506724</v>
       </c>
       <c r="E78" t="n">
-        <v>19.62430811506723</v>
+        <v>19.62430811506724</v>
       </c>
       <c r="F78" t="n">
         <v>25.65964912280701</v>
@@ -39568,10 +39568,10 @@
         <v>25.65964912280701</v>
       </c>
       <c r="D79" t="n">
-        <v>19.62430811506723</v>
+        <v>19.62430811506724</v>
       </c>
       <c r="E79" t="n">
-        <v>19.62430811506723</v>
+        <v>19.62430811506724</v>
       </c>
       <c r="F79" t="n">
         <v>25.65964912280701</v>
@@ -39595,10 +39595,10 @@
         <v>25.65964912280701</v>
       </c>
       <c r="D80" t="n">
-        <v>19.62430811506723</v>
+        <v>19.62430811506724</v>
       </c>
       <c r="E80" t="n">
-        <v>19.62430811506723</v>
+        <v>19.62430811506724</v>
       </c>
       <c r="F80" t="n">
         <v>25.65964912280701</v>
@@ -39622,10 +39622,10 @@
         <v>25.65964912280701</v>
       </c>
       <c r="D81" t="n">
-        <v>19.62430811506723</v>
+        <v>19.62430811506724</v>
       </c>
       <c r="E81" t="n">
-        <v>19.62430811506723</v>
+        <v>19.62430811506724</v>
       </c>
       <c r="F81" t="n">
         <v>25.65964912280701</v>
@@ -40132,16 +40132,16 @@
         <v>77.64667182662539</v>
       </c>
       <c r="D2" t="n">
-        <v>24.25839646159726</v>
+        <v>24.25839646159725</v>
       </c>
       <c r="E2" t="n">
-        <v>24.25839646159726</v>
+        <v>24.25839646159725</v>
       </c>
       <c r="F2" t="n">
         <v>77.64667182662539</v>
       </c>
       <c r="G2" t="n">
-        <v>3.20081634206719</v>
+        <v>3.200816342067191</v>
       </c>
     </row>
     <row r="3">
@@ -40159,16 +40159,16 @@
         <v>77.64667182662539</v>
       </c>
       <c r="D3" t="n">
-        <v>24.25839646159726</v>
+        <v>24.25839646159725</v>
       </c>
       <c r="E3" t="n">
-        <v>24.25839646159726</v>
+        <v>24.25839646159725</v>
       </c>
       <c r="F3" t="n">
         <v>77.64667182662539</v>
       </c>
       <c r="G3" t="n">
-        <v>3.20081634206719</v>
+        <v>3.200816342067191</v>
       </c>
     </row>
     <row r="4">
@@ -40186,16 +40186,16 @@
         <v>77.64667182662539</v>
       </c>
       <c r="D4" t="n">
-        <v>24.25839646159726</v>
+        <v>24.25839646159725</v>
       </c>
       <c r="E4" t="n">
-        <v>24.25839646159726</v>
+        <v>24.25839646159725</v>
       </c>
       <c r="F4" t="n">
         <v>77.64667182662539</v>
       </c>
       <c r="G4" t="n">
-        <v>3.20081634206719</v>
+        <v>3.200816342067191</v>
       </c>
     </row>
     <row r="5">
@@ -40213,16 +40213,16 @@
         <v>77.64667182662539</v>
       </c>
       <c r="D5" t="n">
-        <v>24.25839646159726</v>
+        <v>24.25839646159725</v>
       </c>
       <c r="E5" t="n">
-        <v>24.25839646159726</v>
+        <v>24.25839646159725</v>
       </c>
       <c r="F5" t="n">
         <v>77.64667182662539</v>
       </c>
       <c r="G5" t="n">
-        <v>3.20081634206719</v>
+        <v>3.200816342067191</v>
       </c>
     </row>
     <row r="6">
@@ -41212,16 +41212,16 @@
         <v>77.64667182662539</v>
       </c>
       <c r="D42" t="n">
-        <v>24.25839646159726</v>
+        <v>24.25839646159725</v>
       </c>
       <c r="E42" t="n">
-        <v>24.25839646159726</v>
+        <v>24.25839646159725</v>
       </c>
       <c r="F42" t="n">
         <v>77.64667182662539</v>
       </c>
       <c r="G42" t="n">
-        <v>3.20081634206719</v>
+        <v>3.200816342067191</v>
       </c>
     </row>
     <row r="43">
@@ -41239,16 +41239,16 @@
         <v>77.64667182662539</v>
       </c>
       <c r="D43" t="n">
-        <v>24.25839646159726</v>
+        <v>24.25839646159725</v>
       </c>
       <c r="E43" t="n">
-        <v>24.25839646159726</v>
+        <v>24.25839646159725</v>
       </c>
       <c r="F43" t="n">
         <v>77.64667182662539</v>
       </c>
       <c r="G43" t="n">
-        <v>3.20081634206719</v>
+        <v>3.200816342067191</v>
       </c>
     </row>
     <row r="44">
@@ -41266,16 +41266,16 @@
         <v>77.64667182662539</v>
       </c>
       <c r="D44" t="n">
-        <v>24.25839646159726</v>
+        <v>24.25839646159725</v>
       </c>
       <c r="E44" t="n">
-        <v>24.25839646159726</v>
+        <v>24.25839646159725</v>
       </c>
       <c r="F44" t="n">
         <v>77.64667182662539</v>
       </c>
       <c r="G44" t="n">
-        <v>3.20081634206719</v>
+        <v>3.200816342067191</v>
       </c>
     </row>
     <row r="45">
@@ -41293,16 +41293,16 @@
         <v>77.64667182662539</v>
       </c>
       <c r="D45" t="n">
-        <v>24.25839646159726</v>
+        <v>24.25839646159725</v>
       </c>
       <c r="E45" t="n">
-        <v>24.25839646159726</v>
+        <v>24.25839646159725</v>
       </c>
       <c r="F45" t="n">
         <v>77.64667182662539</v>
       </c>
       <c r="G45" t="n">
-        <v>3.20081634206719</v>
+        <v>3.200816342067191</v>
       </c>
     </row>
     <row r="46">
@@ -41320,16 +41320,16 @@
         <v>77.64667182662539</v>
       </c>
       <c r="D46" t="n">
-        <v>24.25839646159726</v>
+        <v>24.25839646159725</v>
       </c>
       <c r="E46" t="n">
-        <v>24.25839646159726</v>
+        <v>24.25839646159725</v>
       </c>
       <c r="F46" t="n">
         <v>77.64667182662539</v>
       </c>
       <c r="G46" t="n">
-        <v>3.20081634206719</v>
+        <v>3.200816342067191</v>
       </c>
     </row>
     <row r="47">
@@ -41347,16 +41347,16 @@
         <v>77.64667182662539</v>
       </c>
       <c r="D47" t="n">
-        <v>24.25839646159726</v>
+        <v>24.25839646159725</v>
       </c>
       <c r="E47" t="n">
-        <v>24.25839646159726</v>
+        <v>24.25839646159725</v>
       </c>
       <c r="F47" t="n">
         <v>77.64667182662539</v>
       </c>
       <c r="G47" t="n">
-        <v>3.20081634206719</v>
+        <v>3.200816342067191</v>
       </c>
     </row>
     <row r="48">
@@ -41374,16 +41374,16 @@
         <v>77.64667182662539</v>
       </c>
       <c r="D48" t="n">
-        <v>24.25839646159726</v>
+        <v>24.25839646159725</v>
       </c>
       <c r="E48" t="n">
-        <v>24.25839646159726</v>
+        <v>24.25839646159725</v>
       </c>
       <c r="F48" t="n">
         <v>77.64667182662539</v>
       </c>
       <c r="G48" t="n">
-        <v>3.20081634206719</v>
+        <v>3.200816342067191</v>
       </c>
     </row>
     <row r="49">
@@ -41401,16 +41401,16 @@
         <v>77.64667182662539</v>
       </c>
       <c r="D49" t="n">
-        <v>24.25839646159726</v>
+        <v>24.25839646159725</v>
       </c>
       <c r="E49" t="n">
-        <v>24.25839646159726</v>
+        <v>24.25839646159725</v>
       </c>
       <c r="F49" t="n">
         <v>77.64667182662539</v>
       </c>
       <c r="G49" t="n">
-        <v>3.20081634206719</v>
+        <v>3.200816342067191</v>
       </c>
     </row>
     <row r="50">
@@ -41428,16 +41428,16 @@
         <v>77.64667182662539</v>
       </c>
       <c r="D50" t="n">
-        <v>24.25839646159726</v>
+        <v>24.25839646159725</v>
       </c>
       <c r="E50" t="n">
-        <v>24.25839646159726</v>
+        <v>24.25839646159725</v>
       </c>
       <c r="F50" t="n">
         <v>77.64667182662539</v>
       </c>
       <c r="G50" t="n">
-        <v>3.20081634206719</v>
+        <v>3.200816342067191</v>
       </c>
     </row>
     <row r="51">
@@ -41455,16 +41455,16 @@
         <v>77.64667182662539</v>
       </c>
       <c r="D51" t="n">
-        <v>24.25839646159726</v>
+        <v>24.25839646159725</v>
       </c>
       <c r="E51" t="n">
-        <v>24.25839646159726</v>
+        <v>24.25839646159725</v>
       </c>
       <c r="F51" t="n">
         <v>77.64667182662539</v>
       </c>
       <c r="G51" t="n">
-        <v>3.20081634206719</v>
+        <v>3.200816342067191</v>
       </c>
     </row>
     <row r="52">
@@ -41482,16 +41482,16 @@
         <v>77.64667182662539</v>
       </c>
       <c r="D52" t="n">
-        <v>24.25839646159726</v>
+        <v>24.25839646159725</v>
       </c>
       <c r="E52" t="n">
-        <v>24.25839646159726</v>
+        <v>24.25839646159725</v>
       </c>
       <c r="F52" t="n">
         <v>77.64667182662539</v>
       </c>
       <c r="G52" t="n">
-        <v>3.20081634206719</v>
+        <v>3.200816342067191</v>
       </c>
     </row>
     <row r="53">
@@ -41509,16 +41509,16 @@
         <v>77.64667182662539</v>
       </c>
       <c r="D53" t="n">
-        <v>24.25839646159726</v>
+        <v>24.25839646159725</v>
       </c>
       <c r="E53" t="n">
-        <v>24.25839646159726</v>
+        <v>24.25839646159725</v>
       </c>
       <c r="F53" t="n">
         <v>77.64667182662539</v>
       </c>
       <c r="G53" t="n">
-        <v>3.20081634206719</v>
+        <v>3.200816342067191</v>
       </c>
     </row>
     <row r="54">
@@ -41536,16 +41536,16 @@
         <v>77.64667182662539</v>
       </c>
       <c r="D54" t="n">
-        <v>24.25839646159726</v>
+        <v>24.25839646159725</v>
       </c>
       <c r="E54" t="n">
-        <v>24.25839646159726</v>
+        <v>24.25839646159725</v>
       </c>
       <c r="F54" t="n">
         <v>77.64667182662539</v>
       </c>
       <c r="G54" t="n">
-        <v>3.20081634206719</v>
+        <v>3.200816342067191</v>
       </c>
     </row>
     <row r="55">
@@ -41563,16 +41563,16 @@
         <v>77.64667182662539</v>
       </c>
       <c r="D55" t="n">
-        <v>24.25839646159726</v>
+        <v>24.25839646159725</v>
       </c>
       <c r="E55" t="n">
-        <v>24.25839646159726</v>
+        <v>24.25839646159725</v>
       </c>
       <c r="F55" t="n">
         <v>77.64667182662539</v>
       </c>
       <c r="G55" t="n">
-        <v>3.20081634206719</v>
+        <v>3.200816342067191</v>
       </c>
     </row>
     <row r="56">
@@ -41590,16 +41590,16 @@
         <v>77.64667182662539</v>
       </c>
       <c r="D56" t="n">
-        <v>24.25839646159726</v>
+        <v>24.25839646159725</v>
       </c>
       <c r="E56" t="n">
-        <v>24.25839646159726</v>
+        <v>24.25839646159725</v>
       </c>
       <c r="F56" t="n">
         <v>77.64667182662539</v>
       </c>
       <c r="G56" t="n">
-        <v>3.20081634206719</v>
+        <v>3.200816342067191</v>
       </c>
     </row>
     <row r="57">
@@ -41617,16 +41617,16 @@
         <v>77.64667182662539</v>
       </c>
       <c r="D57" t="n">
-        <v>24.25839646159726</v>
+        <v>24.25839646159725</v>
       </c>
       <c r="E57" t="n">
-        <v>24.25839646159726</v>
+        <v>24.25839646159725</v>
       </c>
       <c r="F57" t="n">
         <v>77.64667182662539</v>
       </c>
       <c r="G57" t="n">
-        <v>3.20081634206719</v>
+        <v>3.200816342067191</v>
       </c>
     </row>
     <row r="58">
@@ -41644,16 +41644,16 @@
         <v>77.64667182662539</v>
       </c>
       <c r="D58" t="n">
-        <v>24.25839646159726</v>
+        <v>24.25839646159725</v>
       </c>
       <c r="E58" t="n">
-        <v>24.25839646159726</v>
+        <v>24.25839646159725</v>
       </c>
       <c r="F58" t="n">
         <v>77.64667182662539</v>
       </c>
       <c r="G58" t="n">
-        <v>3.20081634206719</v>
+        <v>3.200816342067191</v>
       </c>
     </row>
     <row r="59">
@@ -41671,16 +41671,16 @@
         <v>77.64667182662539</v>
       </c>
       <c r="D59" t="n">
-        <v>24.25839646159726</v>
+        <v>24.25839646159725</v>
       </c>
       <c r="E59" t="n">
-        <v>24.25839646159726</v>
+        <v>24.25839646159725</v>
       </c>
       <c r="F59" t="n">
         <v>77.64667182662539</v>
       </c>
       <c r="G59" t="n">
-        <v>3.20081634206719</v>
+        <v>3.200816342067191</v>
       </c>
     </row>
     <row r="60">
@@ -41698,16 +41698,16 @@
         <v>77.64667182662539</v>
       </c>
       <c r="D60" t="n">
-        <v>24.25839646159726</v>
+        <v>24.25839646159725</v>
       </c>
       <c r="E60" t="n">
-        <v>24.25839646159726</v>
+        <v>24.25839646159725</v>
       </c>
       <c r="F60" t="n">
         <v>77.64667182662539</v>
       </c>
       <c r="G60" t="n">
-        <v>3.20081634206719</v>
+        <v>3.200816342067191</v>
       </c>
     </row>
     <row r="61">
@@ -41725,16 +41725,16 @@
         <v>77.64667182662539</v>
       </c>
       <c r="D61" t="n">
-        <v>24.25839646159726</v>
+        <v>24.25839646159725</v>
       </c>
       <c r="E61" t="n">
-        <v>24.25839646159726</v>
+        <v>24.25839646159725</v>
       </c>
       <c r="F61" t="n">
         <v>77.64667182662539</v>
       </c>
       <c r="G61" t="n">
-        <v>3.20081634206719</v>
+        <v>3.200816342067191</v>
       </c>
     </row>
     <row r="62">
@@ -41752,16 +41752,16 @@
         <v>77.64667182662539</v>
       </c>
       <c r="D62" t="n">
-        <v>24.25839646159726</v>
+        <v>24.25839646159725</v>
       </c>
       <c r="E62" t="n">
-        <v>24.25839646159726</v>
+        <v>24.25839646159725</v>
       </c>
       <c r="F62" t="n">
         <v>77.64667182662539</v>
       </c>
       <c r="G62" t="n">
-        <v>3.20081634206719</v>
+        <v>3.200816342067191</v>
       </c>
     </row>
     <row r="63">
@@ -41779,16 +41779,16 @@
         <v>77.64667182662539</v>
       </c>
       <c r="D63" t="n">
-        <v>24.25839646159726</v>
+        <v>24.25839646159725</v>
       </c>
       <c r="E63" t="n">
-        <v>24.25839646159726</v>
+        <v>24.25839646159725</v>
       </c>
       <c r="F63" t="n">
         <v>77.64667182662539</v>
       </c>
       <c r="G63" t="n">
-        <v>3.20081634206719</v>
+        <v>3.200816342067191</v>
       </c>
     </row>
     <row r="64">
@@ -41806,16 +41806,16 @@
         <v>77.64667182662539</v>
       </c>
       <c r="D64" t="n">
-        <v>24.25839646159726</v>
+        <v>24.25839646159725</v>
       </c>
       <c r="E64" t="n">
-        <v>24.25839646159726</v>
+        <v>24.25839646159725</v>
       </c>
       <c r="F64" t="n">
         <v>77.64667182662539</v>
       </c>
       <c r="G64" t="n">
-        <v>3.20081634206719</v>
+        <v>3.200816342067191</v>
       </c>
     </row>
     <row r="65">
@@ -41833,16 +41833,16 @@
         <v>77.64667182662539</v>
       </c>
       <c r="D65" t="n">
-        <v>24.25839646159726</v>
+        <v>24.25839646159725</v>
       </c>
       <c r="E65" t="n">
-        <v>24.25839646159726</v>
+        <v>24.25839646159725</v>
       </c>
       <c r="F65" t="n">
         <v>77.64667182662539</v>
       </c>
       <c r="G65" t="n">
-        <v>3.20081634206719</v>
+        <v>3.200816342067191</v>
       </c>
     </row>
     <row r="66">
@@ -41860,16 +41860,16 @@
         <v>77.64667182662539</v>
       </c>
       <c r="D66" t="n">
-        <v>24.25839646159726</v>
+        <v>24.25839646159725</v>
       </c>
       <c r="E66" t="n">
-        <v>24.25839646159726</v>
+        <v>24.25839646159725</v>
       </c>
       <c r="F66" t="n">
         <v>77.64667182662539</v>
       </c>
       <c r="G66" t="n">
-        <v>3.20081634206719</v>
+        <v>3.200816342067191</v>
       </c>
     </row>
     <row r="67">
@@ -41887,16 +41887,16 @@
         <v>77.64667182662539</v>
       </c>
       <c r="D67" t="n">
-        <v>24.25839646159726</v>
+        <v>24.25839646159725</v>
       </c>
       <c r="E67" t="n">
-        <v>24.25839646159726</v>
+        <v>24.25839646159725</v>
       </c>
       <c r="F67" t="n">
         <v>77.64667182662539</v>
       </c>
       <c r="G67" t="n">
-        <v>3.20081634206719</v>
+        <v>3.200816342067191</v>
       </c>
     </row>
     <row r="68">
@@ -41914,16 +41914,16 @@
         <v>77.64667182662539</v>
       </c>
       <c r="D68" t="n">
-        <v>24.25839646159726</v>
+        <v>24.25839646159725</v>
       </c>
       <c r="E68" t="n">
-        <v>24.25839646159726</v>
+        <v>24.25839646159725</v>
       </c>
       <c r="F68" t="n">
         <v>77.64667182662539</v>
       </c>
       <c r="G68" t="n">
-        <v>3.20081634206719</v>
+        <v>3.200816342067191</v>
       </c>
     </row>
     <row r="69">
@@ -41941,16 +41941,16 @@
         <v>77.64667182662539</v>
       </c>
       <c r="D69" t="n">
-        <v>24.25839646159726</v>
+        <v>24.25839646159725</v>
       </c>
       <c r="E69" t="n">
-        <v>24.25839646159726</v>
+        <v>24.25839646159725</v>
       </c>
       <c r="F69" t="n">
         <v>77.64667182662539</v>
       </c>
       <c r="G69" t="n">
-        <v>3.20081634206719</v>
+        <v>3.200816342067191</v>
       </c>
     </row>
     <row r="70">
@@ -42880,7 +42880,7 @@
         </is>
       </c>
       <c r="C6" t="n">
-        <v>366.4282030620467</v>
+        <v>366.4282030620468</v>
       </c>
       <c r="D6" t="n">
         <v>23.97820723550419</v>
@@ -42889,7 +42889,7 @@
         <v>23.97820723550419</v>
       </c>
       <c r="F6" t="n">
-        <v>366.4282030620467</v>
+        <v>366.4282030620468</v>
       </c>
       <c r="G6" t="n">
         <v>15.28171808105327</v>
@@ -42907,7 +42907,7 @@
         </is>
       </c>
       <c r="C7" t="n">
-        <v>366.4282030620467</v>
+        <v>366.4282030620468</v>
       </c>
       <c r="D7" t="n">
         <v>23.97820723550419</v>
@@ -42916,7 +42916,7 @@
         <v>23.97820723550419</v>
       </c>
       <c r="F7" t="n">
-        <v>366.4282030620467</v>
+        <v>366.4282030620468</v>
       </c>
       <c r="G7" t="n">
         <v>15.28171808105327</v>
@@ -42934,7 +42934,7 @@
         </is>
       </c>
       <c r="C8" t="n">
-        <v>366.4282030620467</v>
+        <v>366.4282030620468</v>
       </c>
       <c r="D8" t="n">
         <v>23.97820723550419</v>
@@ -42943,7 +42943,7 @@
         <v>23.97820723550419</v>
       </c>
       <c r="F8" t="n">
-        <v>366.4282030620467</v>
+        <v>366.4282030620468</v>
       </c>
       <c r="G8" t="n">
         <v>15.28171808105327</v>
@@ -42961,7 +42961,7 @@
         </is>
       </c>
       <c r="C9" t="n">
-        <v>366.4282030620467</v>
+        <v>366.4282030620468</v>
       </c>
       <c r="D9" t="n">
         <v>23.97820723550419</v>
@@ -42970,7 +42970,7 @@
         <v>23.97820723550419</v>
       </c>
       <c r="F9" t="n">
-        <v>366.4282030620467</v>
+        <v>366.4282030620468</v>
       </c>
       <c r="G9" t="n">
         <v>15.28171808105327</v>
@@ -42988,7 +42988,7 @@
         </is>
       </c>
       <c r="C10" t="n">
-        <v>366.4282030620467</v>
+        <v>366.4282030620468</v>
       </c>
       <c r="D10" t="n">
         <v>23.97820723550419</v>
@@ -42997,7 +42997,7 @@
         <v>23.97820723550419</v>
       </c>
       <c r="F10" t="n">
-        <v>366.4282030620467</v>
+        <v>366.4282030620468</v>
       </c>
       <c r="G10" t="n">
         <v>15.28171808105327</v>
@@ -43015,7 +43015,7 @@
         </is>
       </c>
       <c r="C11" t="n">
-        <v>366.4282030620467</v>
+        <v>366.4282030620468</v>
       </c>
       <c r="D11" t="n">
         <v>23.97820723550419</v>
@@ -43024,7 +43024,7 @@
         <v>23.97820723550419</v>
       </c>
       <c r="F11" t="n">
-        <v>366.4282030620467</v>
+        <v>366.4282030620468</v>
       </c>
       <c r="G11" t="n">
         <v>15.28171808105327</v>
@@ -43042,7 +43042,7 @@
         </is>
       </c>
       <c r="C12" t="n">
-        <v>366.4282030620467</v>
+        <v>366.4282030620468</v>
       </c>
       <c r="D12" t="n">
         <v>23.97820723550419</v>
@@ -43051,7 +43051,7 @@
         <v>23.97820723550419</v>
       </c>
       <c r="F12" t="n">
-        <v>366.4282030620467</v>
+        <v>366.4282030620468</v>
       </c>
       <c r="G12" t="n">
         <v>15.28171808105327</v>
@@ -43069,7 +43069,7 @@
         </is>
       </c>
       <c r="C13" t="n">
-        <v>366.4282030620467</v>
+        <v>366.4282030620468</v>
       </c>
       <c r="D13" t="n">
         <v>23.97820723550419</v>
@@ -43078,7 +43078,7 @@
         <v>23.97820723550419</v>
       </c>
       <c r="F13" t="n">
-        <v>366.4282030620467</v>
+        <v>366.4282030620468</v>
       </c>
       <c r="G13" t="n">
         <v>15.28171808105327</v>
@@ -43096,7 +43096,7 @@
         </is>
       </c>
       <c r="C14" t="n">
-        <v>366.4282030620467</v>
+        <v>366.4282030620468</v>
       </c>
       <c r="D14" t="n">
         <v>23.97820723550419</v>
@@ -43105,7 +43105,7 @@
         <v>23.97820723550419</v>
       </c>
       <c r="F14" t="n">
-        <v>366.4282030620467</v>
+        <v>366.4282030620468</v>
       </c>
       <c r="G14" t="n">
         <v>15.28171808105327</v>
@@ -43123,7 +43123,7 @@
         </is>
       </c>
       <c r="C15" t="n">
-        <v>366.4282030620467</v>
+        <v>366.4282030620468</v>
       </c>
       <c r="D15" t="n">
         <v>23.97820723550419</v>
@@ -43132,7 +43132,7 @@
         <v>23.97820723550419</v>
       </c>
       <c r="F15" t="n">
-        <v>366.4282030620467</v>
+        <v>366.4282030620468</v>
       </c>
       <c r="G15" t="n">
         <v>15.28171808105327</v>
@@ -43150,7 +43150,7 @@
         </is>
       </c>
       <c r="C16" t="n">
-        <v>366.4282030620467</v>
+        <v>366.4282030620468</v>
       </c>
       <c r="D16" t="n">
         <v>23.97820723550419</v>
@@ -43159,7 +43159,7 @@
         <v>23.97820723550419</v>
       </c>
       <c r="F16" t="n">
-        <v>366.4282030620467</v>
+        <v>366.4282030620468</v>
       </c>
       <c r="G16" t="n">
         <v>15.28171808105327</v>
@@ -43177,7 +43177,7 @@
         </is>
       </c>
       <c r="C17" t="n">
-        <v>366.4282030620467</v>
+        <v>366.4282030620468</v>
       </c>
       <c r="D17" t="n">
         <v>23.97820723550419</v>
@@ -43186,7 +43186,7 @@
         <v>23.97820723550419</v>
       </c>
       <c r="F17" t="n">
-        <v>366.4282030620467</v>
+        <v>366.4282030620468</v>
       </c>
       <c r="G17" t="n">
         <v>15.28171808105327</v>
@@ -43204,7 +43204,7 @@
         </is>
       </c>
       <c r="C18" t="n">
-        <v>366.4282030620467</v>
+        <v>366.4282030620468</v>
       </c>
       <c r="D18" t="n">
         <v>23.97820723550419</v>
@@ -43213,7 +43213,7 @@
         <v>23.97820723550419</v>
       </c>
       <c r="F18" t="n">
-        <v>366.4282030620467</v>
+        <v>366.4282030620468</v>
       </c>
       <c r="G18" t="n">
         <v>15.28171808105327</v>
@@ -43231,7 +43231,7 @@
         </is>
       </c>
       <c r="C19" t="n">
-        <v>366.4282030620467</v>
+        <v>366.4282030620468</v>
       </c>
       <c r="D19" t="n">
         <v>23.97820723550419</v>
@@ -43240,7 +43240,7 @@
         <v>23.97820723550419</v>
       </c>
       <c r="F19" t="n">
-        <v>366.4282030620467</v>
+        <v>366.4282030620468</v>
       </c>
       <c r="G19" t="n">
         <v>15.28171808105327</v>
@@ -43258,7 +43258,7 @@
         </is>
       </c>
       <c r="C20" t="n">
-        <v>366.4282030620467</v>
+        <v>366.4282030620468</v>
       </c>
       <c r="D20" t="n">
         <v>23.97820723550419</v>
@@ -43267,7 +43267,7 @@
         <v>23.97820723550419</v>
       </c>
       <c r="F20" t="n">
-        <v>366.4282030620467</v>
+        <v>366.4282030620468</v>
       </c>
       <c r="G20" t="n">
         <v>15.28171808105327</v>
@@ -43285,7 +43285,7 @@
         </is>
       </c>
       <c r="C21" t="n">
-        <v>366.4282030620467</v>
+        <v>366.4282030620468</v>
       </c>
       <c r="D21" t="n">
         <v>23.97820723550419</v>
@@ -43294,7 +43294,7 @@
         <v>23.97820723550419</v>
       </c>
       <c r="F21" t="n">
-        <v>366.4282030620467</v>
+        <v>366.4282030620468</v>
       </c>
       <c r="G21" t="n">
         <v>15.28171808105327</v>
@@ -43312,7 +43312,7 @@
         </is>
       </c>
       <c r="C22" t="n">
-        <v>366.4282030620467</v>
+        <v>366.4282030620468</v>
       </c>
       <c r="D22" t="n">
         <v>23.97820723550419</v>
@@ -43321,7 +43321,7 @@
         <v>23.97820723550419</v>
       </c>
       <c r="F22" t="n">
-        <v>366.4282030620467</v>
+        <v>366.4282030620468</v>
       </c>
       <c r="G22" t="n">
         <v>15.28171808105327</v>
@@ -43339,7 +43339,7 @@
         </is>
       </c>
       <c r="C23" t="n">
-        <v>366.4282030620467</v>
+        <v>366.4282030620468</v>
       </c>
       <c r="D23" t="n">
         <v>23.97820723550419</v>
@@ -43348,7 +43348,7 @@
         <v>23.97820723550419</v>
       </c>
       <c r="F23" t="n">
-        <v>366.4282030620467</v>
+        <v>366.4282030620468</v>
       </c>
       <c r="G23" t="n">
         <v>15.28171808105327</v>
@@ -43366,7 +43366,7 @@
         </is>
       </c>
       <c r="C24" t="n">
-        <v>366.4282030620467</v>
+        <v>366.4282030620468</v>
       </c>
       <c r="D24" t="n">
         <v>23.97820723550419</v>
@@ -43375,7 +43375,7 @@
         <v>23.97820723550419</v>
       </c>
       <c r="F24" t="n">
-        <v>366.4282030620467</v>
+        <v>366.4282030620468</v>
       </c>
       <c r="G24" t="n">
         <v>15.28171808105327</v>
@@ -43393,7 +43393,7 @@
         </is>
       </c>
       <c r="C25" t="n">
-        <v>366.4282030620467</v>
+        <v>366.4282030620468</v>
       </c>
       <c r="D25" t="n">
         <v>23.97820723550419</v>
@@ -43402,7 +43402,7 @@
         <v>23.97820723550419</v>
       </c>
       <c r="F25" t="n">
-        <v>366.4282030620467</v>
+        <v>366.4282030620468</v>
       </c>
       <c r="G25" t="n">
         <v>15.28171808105327</v>
@@ -51352,10 +51352,10 @@
         <v>533.7287899860918</v>
       </c>
       <c r="D26" t="n">
-        <v>24.68235294367199</v>
+        <v>24.682352943672</v>
       </c>
       <c r="E26" t="n">
-        <v>24.68235294367199</v>
+        <v>24.682352943672</v>
       </c>
       <c r="F26" t="n">
         <v>533.7287899860918</v>
@@ -51379,10 +51379,10 @@
         <v>533.7287899860918</v>
       </c>
       <c r="D27" t="n">
-        <v>24.68235294367199</v>
+        <v>24.682352943672</v>
       </c>
       <c r="E27" t="n">
-        <v>24.68235294367199</v>
+        <v>24.682352943672</v>
       </c>
       <c r="F27" t="n">
         <v>533.7287899860918</v>
@@ -51406,10 +51406,10 @@
         <v>533.7287899860918</v>
       </c>
       <c r="D28" t="n">
-        <v>24.68235294367199</v>
+        <v>24.682352943672</v>
       </c>
       <c r="E28" t="n">
-        <v>24.68235294367199</v>
+        <v>24.682352943672</v>
       </c>
       <c r="F28" t="n">
         <v>533.7287899860918</v>
@@ -51433,10 +51433,10 @@
         <v>533.7287899860918</v>
       </c>
       <c r="D29" t="n">
-        <v>24.68235294367199</v>
+        <v>24.682352943672</v>
       </c>
       <c r="E29" t="n">
-        <v>24.68235294367199</v>
+        <v>24.682352943672</v>
       </c>
       <c r="F29" t="n">
         <v>533.7287899860918</v>
@@ -51460,10 +51460,10 @@
         <v>533.7287899860918</v>
       </c>
       <c r="D30" t="n">
-        <v>24.68235294367199</v>
+        <v>24.682352943672</v>
       </c>
       <c r="E30" t="n">
-        <v>24.68235294367199</v>
+        <v>24.682352943672</v>
       </c>
       <c r="F30" t="n">
         <v>533.7287899860918</v>
@@ -51487,10 +51487,10 @@
         <v>533.7287899860918</v>
       </c>
       <c r="D31" t="n">
-        <v>24.68235294367199</v>
+        <v>24.682352943672</v>
       </c>
       <c r="E31" t="n">
-        <v>24.68235294367199</v>
+        <v>24.682352943672</v>
       </c>
       <c r="F31" t="n">
         <v>533.7287899860918</v>
@@ -51514,10 +51514,10 @@
         <v>533.7287899860918</v>
       </c>
       <c r="D32" t="n">
-        <v>24.68235294367199</v>
+        <v>24.682352943672</v>
       </c>
       <c r="E32" t="n">
-        <v>24.68235294367199</v>
+        <v>24.682352943672</v>
       </c>
       <c r="F32" t="n">
         <v>533.7287899860918</v>
@@ -51541,10 +51541,10 @@
         <v>533.7287899860918</v>
       </c>
       <c r="D33" t="n">
-        <v>24.68235294367199</v>
+        <v>24.682352943672</v>
       </c>
       <c r="E33" t="n">
-        <v>24.68235294367199</v>
+        <v>24.682352943672</v>
       </c>
       <c r="F33" t="n">
         <v>533.7287899860918</v>
@@ -51568,10 +51568,10 @@
         <v>533.7287899860918</v>
       </c>
       <c r="D34" t="n">
-        <v>24.68235294367199</v>
+        <v>24.682352943672</v>
       </c>
       <c r="E34" t="n">
-        <v>24.68235294367199</v>
+        <v>24.682352943672</v>
       </c>
       <c r="F34" t="n">
         <v>533.7287899860918</v>
@@ -51595,10 +51595,10 @@
         <v>533.7287899860918</v>
       </c>
       <c r="D35" t="n">
-        <v>24.68235294367199</v>
+        <v>24.682352943672</v>
       </c>
       <c r="E35" t="n">
-        <v>24.68235294367199</v>
+        <v>24.682352943672</v>
       </c>
       <c r="F35" t="n">
         <v>533.7287899860918</v>
@@ -51622,10 +51622,10 @@
         <v>533.7287899860918</v>
       </c>
       <c r="D36" t="n">
-        <v>24.68235294367199</v>
+        <v>24.682352943672</v>
       </c>
       <c r="E36" t="n">
-        <v>24.68235294367199</v>
+        <v>24.682352943672</v>
       </c>
       <c r="F36" t="n">
         <v>533.7287899860918</v>
@@ -51649,10 +51649,10 @@
         <v>533.7287899860918</v>
       </c>
       <c r="D37" t="n">
-        <v>24.68235294367199</v>
+        <v>24.682352943672</v>
       </c>
       <c r="E37" t="n">
-        <v>24.68235294367199</v>
+        <v>24.682352943672</v>
       </c>
       <c r="F37" t="n">
         <v>533.7287899860918</v>
@@ -51676,10 +51676,10 @@
         <v>533.7287899860918</v>
       </c>
       <c r="D38" t="n">
-        <v>24.68235294367199</v>
+        <v>24.682352943672</v>
       </c>
       <c r="E38" t="n">
-        <v>24.68235294367199</v>
+        <v>24.682352943672</v>
       </c>
       <c r="F38" t="n">
         <v>533.7287899860918</v>
@@ -51703,10 +51703,10 @@
         <v>533.7287899860918</v>
       </c>
       <c r="D39" t="n">
-        <v>24.68235294367199</v>
+        <v>24.682352943672</v>
       </c>
       <c r="E39" t="n">
-        <v>24.68235294367199</v>
+        <v>24.682352943672</v>
       </c>
       <c r="F39" t="n">
         <v>533.7287899860918</v>
@@ -51730,10 +51730,10 @@
         <v>533.7287899860918</v>
       </c>
       <c r="D40" t="n">
-        <v>24.68235294367199</v>
+        <v>24.682352943672</v>
       </c>
       <c r="E40" t="n">
-        <v>24.68235294367199</v>
+        <v>24.682352943672</v>
       </c>
       <c r="F40" t="n">
         <v>533.7287899860918</v>
@@ -51757,10 +51757,10 @@
         <v>533.7287899860918</v>
       </c>
       <c r="D41" t="n">
-        <v>24.68235294367199</v>
+        <v>24.682352943672</v>
       </c>
       <c r="E41" t="n">
-        <v>24.68235294367199</v>
+        <v>24.682352943672</v>
       </c>
       <c r="F41" t="n">
         <v>533.7287899860918</v>

</xml_diff>